<commit_message>
minor updates - cleaning, reformatting, etc...
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/CPI_IAF.xlsx
+++ b/Indicator_Gen/config/CPI_IAF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC6CAF0D-8AAE-4F73-AB21-285F32C62284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7901D95-8F4E-4CAE-A549-BFDC9647AB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="7" r:id="rId1"/>
@@ -19,9 +19,6 @@
     <sheet name="BLS_West" sheetId="6" r:id="rId4"/>
     <sheet name="BLS_West monthly" sheetId="8" r:id="rId5"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId6"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,30 +36,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="322">
   <si>
     <t>Year</t>
   </si>
@@ -1022,6 +997,12 @@
   </si>
   <si>
     <t>Jan-2023</t>
+  </si>
+  <si>
+    <t>https://sacog.sharepoint.com/sites/DataDevelopmentMonitoringandSupport/Shared%20Documents/Data%20Developement,%20Monitoring%20and%20Support/RegionalProgressReport/2021%20report/2020Data/ConnectComms/Costs/gas%20cpi_bag_2016_updated%20transit%20fares%20groups.xlsx?web=1</t>
+  </si>
+  <si>
+    <t>IAF_2024</t>
   </si>
 </sst>
 </file>
@@ -1047,7 +1028,7 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Times New Roman"/>
-      <charset val="204"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1077,7 +1058,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1088,6 +1069,12 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1106,254 +1093,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="monthly cpi west"/>
-      <sheetName val="gasoline_CA"/>
-      <sheetName val="gasoline"/>
-      <sheetName val="transit fares"/>
-      <sheetName val="transit fare groups"/>
-      <sheetName val="pivots"/>
-      <sheetName val="vmt_fhwa"/>
-      <sheetName val="Sheet2"/>
-      <sheetName val="names"/>
-      <sheetName val="vehicle fleet mpg"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="12">
-          <cell r="E12">
-            <v>1998</v>
-          </cell>
-          <cell r="R12">
-            <v>164.4</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="E13">
-            <v>1999</v>
-          </cell>
-          <cell r="R13">
-            <v>168.9</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="E14">
-            <v>2000</v>
-          </cell>
-          <cell r="R14">
-            <v>174.8</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="E15">
-            <v>2001</v>
-          </cell>
-          <cell r="R15">
-            <v>181.2</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="E16">
-            <v>2002</v>
-          </cell>
-          <cell r="R16">
-            <v>184.7</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="E17">
-            <v>2003</v>
-          </cell>
-          <cell r="R17">
-            <v>188.6</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="E18">
-            <v>2004</v>
-          </cell>
-          <cell r="R18">
-            <v>193</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="E19">
-            <v>2005</v>
-          </cell>
-          <cell r="R19">
-            <v>198.9</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="E20">
-            <v>2006</v>
-          </cell>
-          <cell r="R20">
-            <v>205.7</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="E21">
-            <v>2007</v>
-          </cell>
-          <cell r="R21">
-            <v>212.23</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="E22">
-            <v>2008</v>
-          </cell>
-          <cell r="R22">
-            <v>219.64599999999999</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="E23">
-            <v>2009</v>
-          </cell>
-          <cell r="R23">
-            <v>218.822</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="E24">
-            <v>2010</v>
-          </cell>
-          <cell r="R24">
-            <v>221.203</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="E25">
-            <v>2011</v>
-          </cell>
-          <cell r="R25">
-            <v>227.48500000000001</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="E26">
-            <v>2012</v>
-          </cell>
-          <cell r="R26">
-            <v>232.376</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="E27">
-            <v>2013</v>
-          </cell>
-          <cell r="R27">
-            <v>235.82400000000001</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="E28">
-            <v>2014</v>
-          </cell>
-          <cell r="R28">
-            <v>240.215</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="E29">
-            <v>2015</v>
-          </cell>
-          <cell r="R29">
-            <v>243.01499999999999</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="E30">
-            <v>2016</v>
-          </cell>
-          <cell r="R30">
-            <v>247.70500000000001</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="E31">
-            <v>2017</v>
-          </cell>
-          <cell r="R31">
-            <v>254.738</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="E32">
-            <v>2018</v>
-          </cell>
-          <cell r="R32">
-            <v>263.26333333333332</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="E33">
-            <v>2019</v>
-          </cell>
-          <cell r="R33">
-            <v>270.34991666666662</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="E34">
-            <v>2020</v>
-          </cell>
-          <cell r="R34">
-            <v>275.05700000000002</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="E35">
-            <v>2021</v>
-          </cell>
-          <cell r="R35">
-            <v>287.49400000000003</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="E36">
-            <v>2022</v>
-          </cell>
-          <cell r="R36">
-            <v>310.50900000000001</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="E37">
-            <v>2023</v>
-          </cell>
-          <cell r="R37">
-            <v>323.834</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="E38">
-            <v>2024</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1643,14 +1382,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8CD831A-DDC6-4E81-BE18-73D43D199F08}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.19921875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="100.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -1658,7 +1397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
@@ -1666,7 +1405,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -1674,12 +1413,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -1697,27 +1439,28 @@
   <dimension ref="A1:N70"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="14" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.59765625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="11.8984375" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="14" width="11.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1"/>
@@ -1733,22 +1476,22 @@
       <c r="A2">
         <v>2023</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="5">
         <v>331.80399999999997</v>
       </c>
-      <c r="C2">
-        <f>$B$2/B2</f>
+      <c r="C2" s="5">
+        <f t="shared" ref="C2:C33" si="0">$B$2/B2</f>
         <v>1</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="5">
         <f>$B$3/B2</f>
         <v>0.96208605080107534</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="5">
         <f>$B$4/B2</f>
         <v>0.89622487974828513</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="5">
         <f>$B$5/B2</f>
         <v>0.85989017612807572</v>
       </c>
@@ -1757,22 +1500,22 @@
       <c r="A3">
         <v>2022</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="5">
         <v>319.22399999999999</v>
       </c>
-      <c r="C3">
-        <f t="shared" ref="C3:C66" si="0">$B$2/B3</f>
+      <c r="C3" s="5">
+        <f t="shared" si="0"/>
         <v>1.0394080645565495</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="5">
         <f t="shared" ref="D3:D66" si="1">$B$3/B3</f>
         <v>1</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="5">
         <f t="shared" ref="E3:E66" si="2">$B$4/B3</f>
         <v>0.9315433676665914</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="5">
         <f t="shared" ref="F3:F66" si="3">$B$5/B3</f>
         <v>0.89377678370047364</v>
       </c>
@@ -1781,22 +1524,22 @@
       <c r="A4">
         <v>2021</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="5">
         <v>297.37099999999998</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="5">
         <f t="shared" si="0"/>
         <v>1.1157913851720578</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="5">
         <f t="shared" si="1"/>
         <v>1.0734873272780467</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="5">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="5">
         <f t="shared" si="3"/>
         <v>0.95945805071779033</v>
       </c>
@@ -1805,22 +1548,22 @@
       <c r="A5">
         <v>2020</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="5">
         <v>285.315</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="5">
         <f t="shared" si="0"/>
         <v>1.1629392075425407</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="5">
         <f t="shared" si="1"/>
         <v>1.118847589506335</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="5">
         <f t="shared" si="2"/>
         <v>1.0422550514343796</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="5">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -1829,22 +1572,22 @@
       <c r="A6">
         <v>2019</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="5">
         <v>280.63799999999998</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="5">
         <f t="shared" si="0"/>
         <v>1.1823202844946159</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="5">
         <f t="shared" si="1"/>
         <v>1.1374938532914289</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="5">
         <f t="shared" si="2"/>
         <v>1.0596248547951455</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="5">
         <f t="shared" si="3"/>
         <v>1.0166655976738717</v>
       </c>
@@ -1853,22 +1596,22 @@
       <c r="A7">
         <v>2018</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="5">
         <v>272.51</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="5">
         <f t="shared" si="0"/>
         <v>1.2175846757917139</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="5">
         <f t="shared" si="1"/>
         <v>1.1714212322483579</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="5">
         <f t="shared" si="2"/>
         <v>1.0912296796447836</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="5">
         <f t="shared" si="3"/>
         <v>1.0469891013173829</v>
       </c>
@@ -1877,22 +1620,22 @@
       <c r="A8">
         <v>2017</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="5">
         <v>262.80200000000002</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="5">
         <f t="shared" si="0"/>
         <v>1.2625626897816604</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="5">
         <f t="shared" si="1"/>
         <v>1.2146939521008211</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="5">
         <f t="shared" si="2"/>
         <v>1.1315400948242402</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="5">
         <f t="shared" si="3"/>
         <v>1.0856652536890889</v>
       </c>
@@ -1901,22 +1644,22 @@
       <c r="A9">
         <v>2016</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="5">
         <v>255.303</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="5">
         <f t="shared" si="0"/>
         <v>1.2996478693944058</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="5">
         <f t="shared" si="1"/>
         <v>1.2503730860976956</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="5">
         <f t="shared" si="2"/>
         <v>1.1647767554631163</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="5">
         <f t="shared" si="3"/>
         <v>1.1175544353180338</v>
       </c>
@@ -1925,22 +1668,22 @@
       <c r="A10">
         <v>2015</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="5">
         <v>249.666</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="5">
         <f t="shared" si="0"/>
         <v>1.3289915326876707</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="5">
         <f t="shared" si="1"/>
         <v>1.2786042152315493</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="5">
         <f t="shared" si="2"/>
         <v>1.1910752765694967</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="5">
         <f t="shared" si="3"/>
         <v>1.1427867631155224</v>
       </c>
@@ -1949,22 +1692,22 @@
       <c r="A11">
         <v>2014</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="5">
         <v>246.05500000000001</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="5">
         <f t="shared" si="0"/>
         <v>1.3484952551258864</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="5">
         <f t="shared" si="1"/>
         <v>1.2973684745280525</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="5">
         <f t="shared" si="2"/>
         <v>1.2085549978663306</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="5">
         <f t="shared" si="3"/>
         <v>1.1595578224380727</v>
       </c>
@@ -1973,22 +1716,22 @@
       <c r="A12">
         <v>2013</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="5">
         <v>241.62299999999999</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="5">
         <f t="shared" si="0"/>
         <v>1.3732301974563679</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="5">
         <f t="shared" si="1"/>
         <v>1.321165617511578</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="5">
         <f t="shared" si="2"/>
         <v>1.2307230685820472</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="5">
         <f t="shared" si="3"/>
         <v>1.1808271563551485</v>
       </c>
@@ -1997,22 +1740,22 @@
       <c r="A13">
         <v>2012</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="5">
         <v>238.155</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="5">
         <f t="shared" si="0"/>
         <v>1.3932270999979004</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="5">
         <f t="shared" si="1"/>
         <v>1.340404358506015</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="5">
         <f t="shared" si="2"/>
         <v>1.2486447901576703</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="5">
         <f t="shared" si="3"/>
         <v>1.1980222964036027</v>
       </c>
@@ -2021,22 +1764,22 @@
       <c r="A14">
         <v>2011</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="5">
         <v>232.93</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="5">
         <f t="shared" si="0"/>
         <v>1.4244794573477009</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="5">
         <f t="shared" si="1"/>
         <v>1.3704718155669084</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="5">
         <f t="shared" si="2"/>
         <v>1.2766539303653457</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="5">
         <f t="shared" si="3"/>
         <v>1.2248958914695403</v>
       </c>
@@ -2045,22 +1788,22 @@
       <c r="A15">
         <v>2010</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="5">
         <v>226.91900000000001</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="5">
         <f t="shared" si="0"/>
         <v>1.4622133889185125</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="5">
         <f t="shared" si="1"/>
         <v>1.4067751047730688</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="5">
         <f t="shared" si="2"/>
         <v>1.3104720186498264</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="5">
         <f t="shared" si="3"/>
         <v>1.2573429285339701</v>
       </c>
@@ -2069,22 +1812,22 @@
       <c r="A16">
         <v>2009</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="5">
         <v>224.11</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="5">
         <f t="shared" si="0"/>
         <v>1.4805408058542677</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="5">
         <f t="shared" si="1"/>
         <v>1.4244076569541742</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="5">
         <f t="shared" si="2"/>
         <v>1.3268975056891703</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="5">
         <f t="shared" si="3"/>
         <v>1.2731024943108293</v>
       </c>
@@ -2093,22 +1836,22 @@
       <c r="A17">
         <v>2008</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="5">
         <v>224.80699999999999</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="5">
         <f t="shared" si="0"/>
         <v>1.4759504819689777</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="5">
         <f t="shared" si="1"/>
         <v>1.4199913703754776</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="5">
         <f t="shared" si="2"/>
         <v>1.3227835432170707</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="5">
         <f t="shared" si="3"/>
         <v>1.2691553198966226</v>
       </c>
@@ -2117,22 +1860,22 @@
       <c r="A18">
         <v>2007</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="5">
         <v>217.42400000000001</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="5">
         <f t="shared" si="0"/>
         <v>1.5260688792405621</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="5">
         <f t="shared" si="1"/>
         <v>1.4682095812789755</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="5">
         <f t="shared" si="2"/>
         <v>1.3677008977849729</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="5">
         <f t="shared" si="3"/>
         <v>1.3122516373537418</v>
       </c>
@@ -2141,22 +1884,22 @@
       <c r="A19">
         <v>2006</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="5">
         <v>210.5</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="5">
         <f t="shared" si="0"/>
         <v>1.5762660332541567</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="5">
         <f t="shared" si="1"/>
         <v>1.516503562945368</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="5">
         <f t="shared" si="2"/>
         <v>1.4126888361045129</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="5">
         <f t="shared" si="3"/>
         <v>1.35541567695962</v>
       </c>
@@ -2165,22 +1908,22 @@
       <c r="A20">
         <v>2005</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="5">
         <v>202.6</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="5">
         <f t="shared" si="0"/>
         <v>1.6377295162882526</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="5">
         <f t="shared" si="1"/>
         <v>1.5756367226061205</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="5">
         <f t="shared" si="2"/>
         <v>1.4677739387956563</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="5">
         <f t="shared" si="3"/>
         <v>1.4082675222112537</v>
       </c>
@@ -2189,22 +1932,22 @@
       <c r="A21">
         <v>2004</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="5">
         <v>195.4</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="5">
         <f t="shared" si="0"/>
         <v>1.6980757420675536</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="5">
         <f t="shared" si="1"/>
         <v>1.633694984646878</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="5">
         <f t="shared" si="2"/>
         <v>1.5218577277379732</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="5">
         <f t="shared" si="3"/>
         <v>1.4601586489252814</v>
       </c>
@@ -2213,22 +1956,22 @@
       <c r="A22">
         <v>2003</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="5">
         <v>190.4</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="5">
         <f t="shared" si="0"/>
         <v>1.7426680672268906</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="5">
         <f t="shared" si="1"/>
         <v>1.676596638655462</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="5">
         <f t="shared" si="2"/>
         <v>1.5618224789915964</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="5">
         <f t="shared" si="3"/>
         <v>1.498503151260504</v>
       </c>
@@ -2237,22 +1980,22 @@
       <c r="A23">
         <v>2002</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="5">
         <v>186.1</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="5">
         <f t="shared" si="0"/>
         <v>1.7829339065018805</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="5">
         <f t="shared" si="1"/>
         <v>1.715335840945728</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="5">
         <f t="shared" si="2"/>
         <v>1.5979097259537882</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="5">
         <f t="shared" si="3"/>
         <v>1.5331273508866201</v>
       </c>
@@ -2261,22 +2004,22 @@
       <c r="A24">
         <v>2001</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="5">
         <v>181.7</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="5">
         <f t="shared" si="0"/>
         <v>1.8261089708310401</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="5">
         <f t="shared" si="1"/>
         <v>1.7568739680792516</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="5">
         <f t="shared" si="2"/>
         <v>1.6366042927903137</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="5">
         <f t="shared" si="3"/>
         <v>1.5702531645569622</v>
       </c>
@@ -2285,22 +2028,22 @@
       <c r="A25">
         <v>2000</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="5">
         <v>174.8</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="5">
         <f t="shared" si="0"/>
         <v>1.8981922196796337</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="5">
         <f t="shared" si="1"/>
         <v>1.8262242562929061</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="5">
         <f t="shared" si="2"/>
         <v>1.70120709382151</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="5">
         <f t="shared" si="3"/>
         <v>1.6322368421052631</v>
       </c>
@@ -2309,22 +2052,22 @@
       <c r="A26">
         <v>1999</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="5">
         <v>168.5</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="5">
         <f t="shared" si="0"/>
         <v>1.9691632047477743</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="5">
         <f t="shared" si="1"/>
         <v>1.8945044510385756</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="5">
         <f t="shared" si="2"/>
         <v>1.7648130563798219</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="5">
         <f t="shared" si="3"/>
         <v>1.6932640949554896</v>
       </c>
@@ -2333,22 +2076,22 @@
       <c r="A27">
         <v>1998</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="5">
         <v>163.69999999999999</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="5">
         <f t="shared" si="0"/>
         <v>2.0269028711056811</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="5">
         <f t="shared" si="1"/>
         <v>1.9500549786194259</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="5">
         <f t="shared" si="2"/>
         <v>1.8165607819181429</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="5">
         <f t="shared" si="3"/>
         <v>1.7429138668295663</v>
       </c>
@@ -2357,22 +2100,22 @@
       <c r="A28">
         <v>1997</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="5">
         <v>160.5</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="5">
         <f t="shared" si="0"/>
         <v>2.0673146417445483</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="5">
         <f t="shared" si="1"/>
         <v>1.9889345794392523</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="5">
         <f t="shared" si="2"/>
         <v>1.8527788161993768</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="5">
         <f t="shared" si="3"/>
         <v>1.777663551401869</v>
       </c>
@@ -2381,22 +2124,22 @@
       <c r="A29">
         <v>1996</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="5">
         <v>157.1</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="5">
         <f t="shared" si="0"/>
         <v>2.1120560152768935</v>
       </c>
-      <c r="D29">
+      <c r="D29" s="5">
         <f t="shared" si="1"/>
         <v>2.0319796308084022</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="5">
         <f t="shared" si="2"/>
         <v>1.8928771483131763</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="5">
         <f t="shared" si="3"/>
         <v>1.8161362189688097</v>
       </c>
@@ -2405,22 +2148,22 @@
       <c r="A30">
         <v>1995</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="5">
         <v>154</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="5">
         <f t="shared" si="0"/>
         <v>2.1545714285714284</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="5">
         <f t="shared" si="1"/>
         <v>2.072883116883117</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="5">
         <f t="shared" si="2"/>
         <v>1.9309805194805194</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="5">
         <f t="shared" si="3"/>
         <v>1.8526948051948051</v>
       </c>
@@ -2429,22 +2172,22 @@
       <c r="A31">
         <v>1994</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="5">
         <v>151.5</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="5">
         <f t="shared" si="0"/>
         <v>2.1901254125412541</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="5">
         <f t="shared" si="1"/>
         <v>2.1070891089108912</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="5">
         <f t="shared" si="2"/>
         <v>1.9628448844884487</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="5">
         <f t="shared" si="3"/>
         <v>1.8832673267326732</v>
       </c>
@@ -2453,22 +2196,22 @@
       <c r="A32">
         <v>1993</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="5">
         <v>149.4</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="5">
         <f t="shared" si="0"/>
         <v>2.2209103078982593</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="5">
         <f t="shared" si="1"/>
         <v>2.1367068273092369</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="5">
         <f t="shared" si="2"/>
         <v>1.9904350736278444</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="5">
         <f t="shared" si="3"/>
         <v>1.9097389558232931</v>
       </c>
@@ -2477,22 +2220,22 @@
       <c r="A33">
         <v>1992</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="5">
         <v>145.6</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="5">
         <f t="shared" si="0"/>
         <v>2.2788736263736262</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="5">
         <f t="shared" si="1"/>
         <v>2.1924725274725274</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="5">
         <f t="shared" si="2"/>
         <v>2.0423832417582415</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="5">
         <f t="shared" si="3"/>
         <v>1.9595810439560439</v>
       </c>
@@ -2501,22 +2244,22 @@
       <c r="A34">
         <v>1991</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="5">
         <v>140.6</v>
       </c>
-      <c r="C34">
-        <f t="shared" si="0"/>
+      <c r="C34" s="5">
+        <f t="shared" ref="C34:C65" si="4">$B$2/B34</f>
         <v>2.3599146514935989</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="5">
         <f t="shared" si="1"/>
         <v>2.2704409672830725</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="5">
         <f t="shared" si="2"/>
         <v>2.1150142247510666</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="5">
         <f t="shared" si="3"/>
         <v>2.0292674253200569</v>
       </c>
@@ -2525,22 +2268,22 @@
       <c r="A35">
         <v>1990</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="5">
         <v>135</v>
       </c>
-      <c r="C35">
-        <f t="shared" si="0"/>
+      <c r="C35" s="5">
+        <f t="shared" si="4"/>
         <v>2.4578074074074072</v>
       </c>
-      <c r="D35">
+      <c r="D35" s="5">
         <f t="shared" si="1"/>
         <v>2.3646222222222222</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="5">
         <f t="shared" si="2"/>
         <v>2.2027481481481481</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="5">
         <f t="shared" si="3"/>
         <v>2.1134444444444442</v>
       </c>
@@ -2549,22 +2292,22 @@
       <c r="A36">
         <v>1989</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="5">
         <v>128</v>
       </c>
-      <c r="C36">
-        <f t="shared" si="0"/>
+      <c r="C36" s="5">
+        <f t="shared" si="4"/>
         <v>2.5922187499999998</v>
       </c>
-      <c r="D36">
+      <c r="D36" s="5">
         <f t="shared" si="1"/>
         <v>2.4939374999999999</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="5">
         <f t="shared" si="2"/>
         <v>2.3232109374999999</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="5">
         <f t="shared" si="3"/>
         <v>2.2290234375</v>
       </c>
@@ -2573,22 +2316,22 @@
       <c r="A37">
         <v>1988</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="5">
         <v>121.9</v>
       </c>
-      <c r="C37">
-        <f t="shared" si="0"/>
+      <c r="C37" s="5">
+        <f t="shared" si="4"/>
         <v>2.7219360131255126</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="5">
         <f t="shared" si="1"/>
         <v>2.6187366694011485</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="5">
         <f t="shared" si="2"/>
         <v>2.439466776045939</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="5">
         <f t="shared" si="3"/>
         <v>2.340566037735849</v>
       </c>
@@ -2597,22 +2340,22 @@
       <c r="A38">
         <v>1987</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="5">
         <v>116.5</v>
       </c>
-      <c r="C38">
-        <f t="shared" si="0"/>
+      <c r="C38" s="5">
+        <f t="shared" si="4"/>
         <v>2.8481030042918452</v>
       </c>
-      <c r="D38">
+      <c r="D38" s="5">
         <f t="shared" si="1"/>
         <v>2.7401201716738197</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="5">
         <f t="shared" si="2"/>
         <v>2.5525407725321885</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="5">
         <f t="shared" si="3"/>
         <v>2.4490557939914162</v>
       </c>
@@ -2621,22 +2364,22 @@
       <c r="A39">
         <v>1986</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="5">
         <v>112</v>
       </c>
-      <c r="C39">
-        <f t="shared" si="0"/>
+      <c r="C39" s="5">
+        <f t="shared" si="4"/>
         <v>2.9625357142857141</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="5">
         <f t="shared" si="1"/>
         <v>2.8502142857142858</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="5">
         <f t="shared" si="2"/>
         <v>2.6550982142857142</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="5">
         <f t="shared" si="3"/>
         <v>2.5474553571428573</v>
       </c>
@@ -2645,22 +2388,22 @@
       <c r="A40">
         <v>1985</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="5">
         <v>108.6</v>
       </c>
-      <c r="C40">
-        <f t="shared" si="0"/>
+      <c r="C40" s="5">
+        <f t="shared" si="4"/>
         <v>3.0552854511970535</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="5">
         <f t="shared" si="1"/>
         <v>2.939447513812155</v>
       </c>
-      <c r="E40">
+      <c r="E40" s="5">
         <f t="shared" si="2"/>
         <v>2.7382228360957641</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="5">
         <f t="shared" si="3"/>
         <v>2.6272099447513813</v>
       </c>
@@ -2669,22 +2412,22 @@
       <c r="A41">
         <v>1984</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="5">
         <v>103.8</v>
       </c>
-      <c r="C41">
-        <f t="shared" si="0"/>
+      <c r="C41" s="5">
+        <f t="shared" si="4"/>
         <v>3.1965703275529864</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="5">
         <f t="shared" si="1"/>
         <v>3.0753757225433525</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="5">
         <f t="shared" si="2"/>
         <v>2.8648458574181115</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="5">
         <f t="shared" si="3"/>
         <v>2.748699421965318</v>
       </c>
@@ -2693,22 +2436,22 @@
       <c r="A42">
         <v>1983</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="5">
         <v>98.9</v>
       </c>
-      <c r="C42">
-        <f t="shared" si="0"/>
+      <c r="C42" s="5">
+        <f t="shared" si="4"/>
         <v>3.3549443882709804</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="5">
         <f t="shared" si="1"/>
         <v>3.2277451971688573</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="5">
         <f t="shared" si="2"/>
         <v>3.0067846309403432</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="5">
         <f t="shared" si="3"/>
         <v>2.8848837209302323</v>
       </c>
@@ -2717,22 +2460,22 @@
       <c r="A43">
         <v>1982</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="5">
         <v>97.3</v>
       </c>
-      <c r="C43">
-        <f t="shared" si="0"/>
+      <c r="C43" s="5">
+        <f t="shared" si="4"/>
         <v>3.4101130524152103</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="5">
         <f t="shared" si="1"/>
         <v>3.2808221993833504</v>
       </c>
-      <c r="E43">
+      <c r="E43" s="5">
         <f t="shared" si="2"/>
         <v>3.0562281603288795</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="5">
         <f t="shared" si="3"/>
         <v>2.9323227132579652</v>
       </c>
@@ -2741,22 +2484,22 @@
       <c r="A44">
         <v>1981</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="5">
         <v>91.4</v>
       </c>
-      <c r="C44">
-        <f t="shared" si="0"/>
+      <c r="C44" s="5">
+        <f t="shared" si="4"/>
         <v>3.6302407002188177</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="5">
         <f t="shared" si="1"/>
         <v>3.492603938730853</v>
       </c>
-      <c r="E44">
+      <c r="E44" s="5">
         <f t="shared" si="2"/>
         <v>3.2535120350109406</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="5">
         <f t="shared" si="3"/>
         <v>3.1216083150984679</v>
       </c>
@@ -2765,22 +2508,22 @@
       <c r="A45">
         <v>1980</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="5">
         <v>82.4</v>
       </c>
-      <c r="C45">
-        <f t="shared" si="0"/>
+      <c r="C45" s="5">
+        <f t="shared" si="4"/>
         <v>4.0267475728155331</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="5">
         <f t="shared" si="1"/>
         <v>3.874077669902912</v>
       </c>
-      <c r="E45">
+      <c r="E45" s="5">
         <f t="shared" si="2"/>
         <v>3.6088713592233006</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="5">
         <f t="shared" si="3"/>
         <v>3.4625606796116504</v>
       </c>
@@ -2789,22 +2532,22 @@
       <c r="A46">
         <v>1979</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="5">
         <v>71.3</v>
       </c>
-      <c r="C46">
-        <f t="shared" si="0"/>
+      <c r="C46" s="5">
+        <f t="shared" si="4"/>
         <v>4.6536325385694246</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="5">
         <f t="shared" si="1"/>
         <v>4.4771949509116409</v>
       </c>
-      <c r="E46">
+      <c r="E46" s="5">
         <f t="shared" si="2"/>
         <v>4.1707012622720896</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="5">
         <f t="shared" si="3"/>
         <v>4.0016129032258068</v>
       </c>
@@ -2813,22 +2556,22 @@
       <c r="A47">
         <v>1978</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="5">
         <v>64.400000000000006</v>
       </c>
-      <c r="C47">
-        <f t="shared" si="0"/>
+      <c r="C47" s="5">
+        <f t="shared" si="4"/>
         <v>5.1522360248447194</v>
       </c>
-      <c r="D47">
+      <c r="D47" s="5">
         <f t="shared" si="1"/>
         <v>4.9568944099378873</v>
       </c>
-      <c r="E47">
+      <c r="E47" s="5">
         <f t="shared" si="2"/>
         <v>4.6175621118012415</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="5">
         <f t="shared" si="3"/>
         <v>4.430357142857142</v>
       </c>
@@ -2837,22 +2580,22 @@
       <c r="A48">
         <v>1977</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="5">
         <v>59.5</v>
       </c>
-      <c r="C48">
-        <f t="shared" si="0"/>
+      <c r="C48" s="5">
+        <f t="shared" si="4"/>
         <v>5.5765378151260503</v>
       </c>
-      <c r="D48">
+      <c r="D48" s="5">
         <f t="shared" si="1"/>
         <v>5.3651092436974785</v>
       </c>
-      <c r="E48">
+      <c r="E48" s="5">
         <f t="shared" si="2"/>
         <v>4.9978319327731091</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="5">
         <f t="shared" si="3"/>
         <v>4.7952100840336138</v>
       </c>
@@ -2861,22 +2604,22 @@
       <c r="A49">
         <v>1976</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="5">
         <v>55.6</v>
       </c>
-      <c r="C49">
-        <f t="shared" si="0"/>
+      <c r="C49" s="5">
+        <f t="shared" si="4"/>
         <v>5.9676978417266184</v>
       </c>
-      <c r="D49">
+      <c r="D49" s="5">
         <f t="shared" si="1"/>
         <v>5.741438848920863</v>
       </c>
-      <c r="E49">
+      <c r="E49" s="5">
         <f t="shared" si="2"/>
         <v>5.3483992805755394</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="5">
         <f t="shared" si="3"/>
         <v>5.1315647482014386</v>
       </c>
@@ -2885,22 +2628,22 @@
       <c r="A50">
         <v>1975</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="5">
         <v>52.3</v>
       </c>
-      <c r="C50">
-        <f t="shared" si="0"/>
+      <c r="C50" s="5">
+        <f t="shared" si="4"/>
         <v>6.3442447418738048</v>
       </c>
-      <c r="D50">
+      <c r="D50" s="5">
         <f t="shared" si="1"/>
         <v>6.1037093690248572</v>
       </c>
-      <c r="E50">
+      <c r="E50" s="5">
         <f t="shared" si="2"/>
         <v>5.6858699808795414</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="5">
         <f t="shared" si="3"/>
         <v>5.4553537284894844</v>
       </c>
@@ -2909,22 +2652,22 @@
       <c r="A51">
         <v>1974</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="5">
         <v>47.4</v>
       </c>
-      <c r="C51">
-        <f t="shared" si="0"/>
+      <c r="C51" s="5">
+        <f t="shared" si="4"/>
         <v>7.0000843881856536</v>
       </c>
-      <c r="D51">
+      <c r="D51" s="5">
         <f t="shared" si="1"/>
         <v>6.7346835443037971</v>
       </c>
-      <c r="E51">
+      <c r="E51" s="5">
         <f t="shared" si="2"/>
         <v>6.2736497890295357</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="5">
         <f t="shared" si="3"/>
         <v>6.0193037974683543</v>
       </c>
@@ -2933,22 +2676,22 @@
       <c r="A52">
         <v>1973</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="5">
         <v>43</v>
       </c>
-      <c r="C52">
-        <f t="shared" si="0"/>
+      <c r="C52" s="5">
+        <f t="shared" si="4"/>
         <v>7.7163720930232556</v>
       </c>
-      <c r="D52">
+      <c r="D52" s="5">
         <f t="shared" si="1"/>
         <v>7.4238139534883718</v>
       </c>
-      <c r="E52">
+      <c r="E52" s="5">
         <f t="shared" si="2"/>
         <v>6.9156046511627904</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="5">
         <f t="shared" si="3"/>
         <v>6.6352325581395348</v>
       </c>
@@ -2957,22 +2700,22 @@
       <c r="A53">
         <v>1972</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="5">
         <v>40.6</v>
       </c>
-      <c r="C53">
-        <f t="shared" si="0"/>
+      <c r="C53" s="5">
+        <f t="shared" si="4"/>
         <v>8.1725123152709358</v>
       </c>
-      <c r="D53">
+      <c r="D53" s="5">
         <f t="shared" si="1"/>
         <v>7.8626600985221673</v>
       </c>
-      <c r="E53">
+      <c r="E53" s="5">
         <f t="shared" si="2"/>
         <v>7.3244088669950731</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="5">
         <f t="shared" si="3"/>
         <v>7.0274630541871916</v>
       </c>
@@ -2981,22 +2724,22 @@
       <c r="A54">
         <v>1971</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="5">
         <v>39.299999999999997</v>
       </c>
-      <c r="C54">
-        <f t="shared" si="0"/>
+      <c r="C54" s="5">
+        <f t="shared" si="4"/>
         <v>8.4428498727735377</v>
       </c>
-      <c r="D54">
+      <c r="D54" s="5">
         <f t="shared" si="1"/>
         <v>8.1227480916030537</v>
       </c>
-      <c r="E54">
+      <c r="E54" s="5">
         <f t="shared" si="2"/>
         <v>7.5666921119592878</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="5">
         <f t="shared" si="3"/>
         <v>7.2599236641221383</v>
       </c>
@@ -3005,22 +2748,22 @@
       <c r="A55">
         <v>1970</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="5">
         <v>37.9</v>
       </c>
-      <c r="C55">
-        <f t="shared" si="0"/>
+      <c r="C55" s="5">
+        <f t="shared" si="4"/>
         <v>8.7547229551451178</v>
       </c>
-      <c r="D55">
+      <c r="D55" s="5">
         <f t="shared" si="1"/>
         <v>8.4227968337730879</v>
       </c>
-      <c r="E55">
+      <c r="E55" s="5">
         <f t="shared" si="2"/>
         <v>7.8462005277044851</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="5">
         <f t="shared" si="3"/>
         <v>7.5281002638522434</v>
       </c>
@@ -3029,22 +2772,22 @@
       <c r="A56">
         <v>1969</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="5">
         <v>36.1</v>
       </c>
-      <c r="C56">
-        <f t="shared" si="0"/>
+      <c r="C56" s="5">
+        <f t="shared" si="4"/>
         <v>9.1912465373961201</v>
       </c>
-      <c r="D56">
+      <c r="D56" s="5">
         <f t="shared" si="1"/>
         <v>8.8427700831024918</v>
       </c>
-      <c r="E56">
+      <c r="E56" s="5">
         <f t="shared" si="2"/>
         <v>8.2374238227146801</v>
       </c>
-      <c r="F56">
+      <c r="F56" s="5">
         <f t="shared" si="3"/>
         <v>7.9034626038781157</v>
       </c>
@@ -3053,22 +2796,22 @@
       <c r="A57">
         <v>1968</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="5">
         <v>34.4</v>
       </c>
-      <c r="C57">
-        <f t="shared" si="0"/>
+      <c r="C57" s="5">
+        <f t="shared" si="4"/>
         <v>9.6454651162790697</v>
       </c>
-      <c r="D57">
+      <c r="D57" s="5">
         <f t="shared" si="1"/>
         <v>9.2797674418604643</v>
       </c>
-      <c r="E57">
+      <c r="E57" s="5">
         <f t="shared" si="2"/>
         <v>8.6445058139534883</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="5">
         <f t="shared" si="3"/>
         <v>8.2940406976744185</v>
       </c>
@@ -3077,22 +2820,22 @@
       <c r="A58">
         <v>1967</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="5">
         <v>33</v>
       </c>
-      <c r="C58">
-        <f t="shared" si="0"/>
+      <c r="C58" s="5">
+        <f t="shared" si="4"/>
         <v>10.054666666666666</v>
       </c>
-      <c r="D58">
+      <c r="D58" s="5">
         <f t="shared" si="1"/>
         <v>9.6734545454545451</v>
       </c>
-      <c r="E58">
+      <c r="E58" s="5">
         <f t="shared" si="2"/>
         <v>9.0112424242424236</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="5">
         <f t="shared" si="3"/>
         <v>8.6459090909090914</v>
       </c>
@@ -3101,22 +2844,22 @@
       <c r="A59">
         <v>1966</v>
       </c>
-      <c r="B59">
+      <c r="B59" s="5">
         <v>32.200000000000003</v>
       </c>
-      <c r="C59">
-        <f t="shared" si="0"/>
+      <c r="C59" s="5">
+        <f t="shared" si="4"/>
         <v>10.304472049689439</v>
       </c>
-      <c r="D59">
+      <c r="D59" s="5">
         <f t="shared" si="1"/>
         <v>9.9137888198757746</v>
       </c>
-      <c r="E59">
+      <c r="E59" s="5">
         <f t="shared" si="2"/>
         <v>9.2351242236024831</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="5">
         <f t="shared" si="3"/>
         <v>8.860714285714284</v>
       </c>
@@ -3125,22 +2868,22 @@
       <c r="A60">
         <v>1965</v>
       </c>
-      <c r="B60">
+      <c r="B60" s="5">
         <v>31.5</v>
       </c>
-      <c r="C60">
-        <f t="shared" si="0"/>
+      <c r="C60" s="5">
+        <f t="shared" si="4"/>
         <v>10.533460317460317</v>
       </c>
-      <c r="D60">
+      <c r="D60" s="5">
         <f t="shared" si="1"/>
         <v>10.134095238095238</v>
       </c>
-      <c r="E60">
+      <c r="E60" s="5">
         <f t="shared" si="2"/>
         <v>9.4403492063492056</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="5">
         <f t="shared" si="3"/>
         <v>9.0576190476190472</v>
       </c>
@@ -3149,22 +2892,22 @@
       <c r="A61">
         <v>1964</v>
       </c>
-      <c r="B61">
+      <c r="B61" s="5">
         <v>31</v>
       </c>
-      <c r="C61">
-        <f t="shared" si="0"/>
+      <c r="C61" s="5">
+        <f t="shared" si="4"/>
         <v>10.703354838709677</v>
       </c>
-      <c r="D61">
+      <c r="D61" s="5">
         <f t="shared" si="1"/>
         <v>10.297548387096773</v>
       </c>
-      <c r="E61">
+      <c r="E61" s="5">
         <f t="shared" si="2"/>
         <v>9.5926129032258061</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="5">
         <f t="shared" si="3"/>
         <v>9.2037096774193543</v>
       </c>
@@ -3173,22 +2916,22 @@
       <c r="A62">
         <v>1963</v>
       </c>
-      <c r="B62">
+      <c r="B62" s="5">
         <v>30.4</v>
       </c>
-      <c r="C62">
-        <f t="shared" si="0"/>
+      <c r="C62" s="5">
+        <f t="shared" si="4"/>
         <v>10.914605263157894</v>
       </c>
-      <c r="D62">
+      <c r="D62" s="5">
         <f t="shared" si="1"/>
         <v>10.500789473684211</v>
       </c>
-      <c r="E62">
+      <c r="E62" s="5">
         <f t="shared" si="2"/>
         <v>9.7819407894736834</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="5">
         <f t="shared" si="3"/>
         <v>9.3853618421052634</v>
       </c>
@@ -3197,22 +2940,22 @@
       <c r="A63">
         <v>1962</v>
       </c>
-      <c r="B63">
+      <c r="B63" s="5">
         <v>29.9</v>
       </c>
-      <c r="C63">
-        <f t="shared" si="0"/>
+      <c r="C63" s="5">
+        <f t="shared" si="4"/>
         <v>11.097123745819397</v>
       </c>
-      <c r="D63">
+      <c r="D63" s="5">
         <f t="shared" si="1"/>
         <v>10.67638795986622</v>
       </c>
-      <c r="E63">
+      <c r="E63" s="5">
         <f t="shared" si="2"/>
         <v>9.945518394648829</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="5">
         <f t="shared" si="3"/>
         <v>9.542307692307693</v>
       </c>
@@ -3221,22 +2964,22 @@
       <c r="A64">
         <v>1961</v>
       </c>
-      <c r="B64">
+      <c r="B64" s="5">
         <v>29.5</v>
       </c>
-      <c r="C64">
-        <f t="shared" si="0"/>
+      <c r="C64" s="5">
+        <f t="shared" si="4"/>
         <v>11.247593220338983</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="5">
         <f t="shared" si="1"/>
         <v>10.82115254237288</v>
       </c>
-      <c r="E64">
+      <c r="E64" s="5">
         <f t="shared" si="2"/>
         <v>10.080372881355931</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="5">
         <f t="shared" si="3"/>
         <v>9.6716949152542373</v>
       </c>
@@ -3245,22 +2988,22 @@
       <c r="A65">
         <v>1960</v>
       </c>
-      <c r="B65">
+      <c r="B65" s="5">
         <v>29.2</v>
       </c>
-      <c r="C65">
-        <f t="shared" si="0"/>
+      <c r="C65" s="5">
+        <f t="shared" si="4"/>
         <v>11.363150684931506</v>
       </c>
-      <c r="D65">
+      <c r="D65" s="5">
         <f t="shared" si="1"/>
         <v>10.932328767123288</v>
       </c>
-      <c r="E65">
+      <c r="E65" s="5">
         <f t="shared" si="2"/>
         <v>10.183938356164383</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="5">
         <f t="shared" si="3"/>
         <v>9.7710616438356173</v>
       </c>
@@ -3269,22 +3012,22 @@
       <c r="A66">
         <v>1959</v>
       </c>
-      <c r="B66">
+      <c r="B66" s="5">
         <v>28.6</v>
       </c>
-      <c r="C66">
-        <f t="shared" si="0"/>
+      <c r="C66" s="5">
+        <f t="shared" ref="C66:C97" si="5">$B$2/B66</f>
         <v>11.60153846153846</v>
       </c>
-      <c r="D66">
+      <c r="D66" s="5">
         <f t="shared" si="1"/>
         <v>11.161678321678322</v>
       </c>
-      <c r="E66">
+      <c r="E66" s="5">
         <f t="shared" si="2"/>
         <v>10.397587412587411</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="5">
         <f t="shared" si="3"/>
         <v>9.9760489510489503</v>
       </c>
@@ -3293,23 +3036,23 @@
       <c r="A67">
         <v>1958</v>
       </c>
-      <c r="B67">
+      <c r="B67" s="5">
         <v>28.1</v>
       </c>
-      <c r="C67">
-        <f t="shared" ref="C67:C70" si="4">$B$2/B67</f>
+      <c r="C67" s="5">
+        <f t="shared" si="5"/>
         <v>11.807971530249109</v>
       </c>
-      <c r="D67">
-        <f t="shared" ref="D67:D70" si="5">$B$3/B67</f>
+      <c r="D67" s="5">
+        <f t="shared" ref="D67:D70" si="6">$B$3/B67</f>
         <v>11.360284697508895</v>
       </c>
-      <c r="E67">
-        <f t="shared" ref="E67:E70" si="6">$B$4/B67</f>
+      <c r="E67" s="5">
+        <f t="shared" ref="E67:E70" si="7">$B$4/B67</f>
         <v>10.582597864768681</v>
       </c>
-      <c r="F67">
-        <f t="shared" ref="F67:F70" si="7">$B$5/B67</f>
+      <c r="F67" s="5">
+        <f t="shared" ref="F67:F70" si="8">$B$5/B67</f>
         <v>10.153558718861209</v>
       </c>
     </row>
@@ -3317,23 +3060,23 @@
       <c r="A68">
         <v>1957</v>
       </c>
-      <c r="B68">
+      <c r="B68" s="5">
         <v>27.1</v>
       </c>
-      <c r="C68">
-        <f t="shared" si="4"/>
+      <c r="C68" s="5">
+        <f t="shared" si="5"/>
         <v>12.243690036900368</v>
       </c>
-      <c r="D68">
-        <f t="shared" si="5"/>
+      <c r="D68" s="5">
+        <f t="shared" si="6"/>
         <v>11.779483394833948</v>
       </c>
-      <c r="E68">
-        <f t="shared" si="6"/>
+      <c r="E68" s="5">
+        <f t="shared" si="7"/>
         <v>10.973099630996309</v>
       </c>
-      <c r="F68">
-        <f t="shared" si="7"/>
+      <c r="F68" s="5">
+        <f t="shared" si="8"/>
         <v>10.528228782287822</v>
       </c>
     </row>
@@ -3341,23 +3084,23 @@
       <c r="A69">
         <v>1956</v>
       </c>
-      <c r="B69">
+      <c r="B69" s="5">
         <v>26.2</v>
       </c>
-      <c r="C69">
-        <f t="shared" si="4"/>
+      <c r="C69" s="5">
+        <f t="shared" si="5"/>
         <v>12.664274809160304</v>
       </c>
-      <c r="D69">
-        <f t="shared" si="5"/>
+      <c r="D69" s="5">
+        <f t="shared" si="6"/>
         <v>12.18412213740458</v>
       </c>
-      <c r="E69">
-        <f t="shared" si="6"/>
+      <c r="E69" s="5">
+        <f t="shared" si="7"/>
         <v>11.350038167938932</v>
       </c>
-      <c r="F69">
-        <f t="shared" si="7"/>
+      <c r="F69" s="5">
+        <f t="shared" si="8"/>
         <v>10.889885496183206</v>
       </c>
     </row>
@@ -3365,23 +3108,23 @@
       <c r="A70">
         <v>1955</v>
       </c>
-      <c r="B70">
+      <c r="B70" s="5">
         <v>25.7</v>
       </c>
-      <c r="C70">
-        <f t="shared" si="4"/>
+      <c r="C70" s="5">
+        <f t="shared" si="5"/>
         <v>12.910661478599222</v>
       </c>
-      <c r="D70">
-        <f t="shared" si="5"/>
+      <c r="D70" s="5">
+        <f t="shared" si="6"/>
         <v>12.421167315175097</v>
       </c>
-      <c r="E70">
-        <f t="shared" si="6"/>
+      <c r="E70" s="5">
+        <f t="shared" si="7"/>
         <v>11.570856031128404</v>
       </c>
-      <c r="F70">
-        <f t="shared" si="7"/>
+      <c r="F70" s="5">
+        <f t="shared" si="8"/>
         <v>11.101750972762646</v>
       </c>
     </row>
@@ -4534,32 +4277,35 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBBF9ED9-28E1-4BE7-8184-11175FEC6A7E}">
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="6" width="12.8984375" customWidth="1"/>
+    <col min="1" max="1" width="12.8984375" customWidth="1"/>
+    <col min="2" max="7" width="12.8984375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -4567,654 +4313,761 @@
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2023</v>
-      </c>
-      <c r="B2" cm="1">
-        <f t="array" ref="B2">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A2,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>323.834</v>
-      </c>
-      <c r="C2">
+        <v>2024</v>
+      </c>
+      <c r="B2" s="5">
+        <v>332.94499999999999</v>
+      </c>
+      <c r="C2" s="5">
         <f>$B$2/B2</f>
         <v>1</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="5">
         <f>$B$3/B2</f>
-        <v>0.95885237498224407</v>
-      </c>
-      <c r="E2">
-        <f t="shared" ref="E2:E3" si="0">$B$4/B2</f>
-        <v>0.88778201177146321</v>
-      </c>
-      <c r="F2">
-        <f t="shared" ref="F2:F4" si="1">$B$5/B2</f>
-        <v>0.84937653242093181</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0.97263511991470064</v>
+      </c>
+      <c r="E2" s="5">
+        <f>$B$4/B2</f>
+        <v>0.93261349472135047</v>
+      </c>
+      <c r="F2" s="5">
+        <f t="shared" ref="F2:F4" si="0">$B$5/B2</f>
+        <v>0.86348796347745138</v>
+      </c>
+      <c r="G2" s="5">
+        <f t="shared" ref="G2:G5" si="1">$B$6/B2</f>
+        <v>0.82613344546396561</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>2022</v>
-      </c>
-      <c r="B3" cm="1">
-        <f t="array" ref="B3">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A3,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>310.50900000000001</v>
-      </c>
-      <c r="C3">
-        <f t="shared" ref="C3:C27" si="2">$B$2/B3</f>
-        <v>1.0429134099172648</v>
-      </c>
-      <c r="D3">
+        <v>2023</v>
+      </c>
+      <c r="B3" s="5">
+        <v>323.834</v>
+      </c>
+      <c r="C3" s="5">
+        <f t="shared" ref="C3:C28" si="2">$B$2/B3</f>
+        <v>1.0281347851059492</v>
+      </c>
+      <c r="D3" s="5">
         <f>$B$3/B3</f>
         <v>1</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="5">
+        <f>$B$4/B3</f>
+        <v>0.95885237498224407</v>
+      </c>
+      <c r="F3" s="5">
+        <f t="shared" si="0"/>
+        <v>0.88778201177146321</v>
+      </c>
+      <c r="G3" s="5">
+        <f t="shared" si="1"/>
+        <v>0.84937653242093181</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2022</v>
+      </c>
+      <c r="B4" s="5">
+        <v>310.50900000000001</v>
+      </c>
+      <c r="C4" s="5">
+        <f t="shared" si="2"/>
+        <v>1.0722555545893999</v>
+      </c>
+      <c r="D4" s="5">
+        <f t="shared" ref="D4:D28" si="3">$B$3/B4</f>
+        <v>1.0429134099172648</v>
+      </c>
+      <c r="E4" s="5">
+        <f>$B$4/B4</f>
+        <v>1</v>
+      </c>
+      <c r="F4" s="5">
         <f t="shared" si="0"/>
         <v>0.92587976515978609</v>
       </c>
-      <c r="F3">
+      <c r="G4" s="5">
         <f t="shared" si="1"/>
         <v>0.88582617573081623</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>2021</v>
       </c>
-      <c r="B4" cm="1">
-        <f t="array" ref="B4">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A4,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
+      <c r="B5" s="5">
         <v>287.49400000000003</v>
       </c>
-      <c r="C4">
-        <f t="shared" si="2"/>
+      <c r="C5" s="5">
+        <f t="shared" si="2"/>
+        <v>1.1580937341301034</v>
+      </c>
+      <c r="D5" s="5">
+        <f t="shared" si="3"/>
         <v>1.1264026379680967</v>
       </c>
-      <c r="D4">
-        <f t="shared" ref="D4:D27" si="3">$B$3/B4</f>
+      <c r="E5" s="5">
+        <f t="shared" ref="E5:E28" si="4">$B$4/B5</f>
         <v>1.0800538446019743</v>
       </c>
-      <c r="E4">
-        <f>$B$4/B4</f>
+      <c r="F5" s="5">
+        <f>$B$5/B5</f>
         <v>1</v>
       </c>
-      <c r="F4">
+      <c r="G5" s="5">
         <f t="shared" si="1"/>
         <v>0.95673996674713213</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>2020</v>
       </c>
-      <c r="B5" cm="1">
-        <f t="array" ref="B5">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A5,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
+      <c r="B6" s="5">
         <v>275.05700000000002</v>
       </c>
-      <c r="C5">
-        <f t="shared" si="2"/>
+      <c r="C6" s="5">
+        <f t="shared" si="2"/>
+        <v>1.2104581959375693</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="3"/>
         <v>1.1773341525574699</v>
       </c>
-      <c r="D5">
-        <f t="shared" si="3"/>
+      <c r="E6" s="5">
+        <f t="shared" si="4"/>
         <v>1.1288896483274375</v>
       </c>
-      <c r="E5">
-        <f t="shared" ref="E5:E27" si="4">$B$4/B5</f>
+      <c r="F6" s="5">
+        <f t="shared" ref="F6:F28" si="5">$B$5/B6</f>
         <v>1.0452160824847214</v>
       </c>
-      <c r="F5">
-        <f>$B$5/B5</f>
+      <c r="G6" s="5">
+        <f>$B$6/B6</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>2019</v>
       </c>
-      <c r="B6" cm="1">
-        <f t="array" ref="B6">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A6,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
+      <c r="B7" s="5">
         <v>270.34991666666662</v>
       </c>
-      <c r="C6">
-        <f t="shared" si="2"/>
+      <c r="C7" s="5">
+        <f t="shared" si="2"/>
+        <v>1.2315335773175446</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="3"/>
         <v>1.1978328086532302</v>
       </c>
-      <c r="D6">
-        <f t="shared" si="3"/>
+      <c r="E7" s="5">
+        <f t="shared" si="4"/>
         <v>1.1485448334088015</v>
       </c>
-      <c r="E6">
-        <f t="shared" si="4"/>
+      <c r="F7" s="5">
+        <f t="shared" si="5"/>
         <v>1.0634144206320268</v>
       </c>
-      <c r="F6">
-        <f t="shared" ref="F6:F27" si="5">$B$5/B6</f>
+      <c r="G7" s="5">
+        <f t="shared" ref="G7:G28" si="6">$B$6/B7</f>
         <v>1.017411077433906</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>2018</v>
       </c>
-      <c r="B7" cm="1">
-        <f t="array" ref="B7">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A7,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
+      <c r="B8" s="5">
         <v>263.26333333333332</v>
       </c>
-      <c r="C7">
-        <f t="shared" si="2"/>
+      <c r="C8" s="5">
+        <f t="shared" si="2"/>
+        <v>1.2646842831638789</v>
+      </c>
+      <c r="D8" s="5">
+        <f t="shared" si="3"/>
         <v>1.2300763494093367</v>
       </c>
-      <c r="D7">
-        <f t="shared" si="3"/>
+      <c r="E8" s="5">
+        <f t="shared" si="4"/>
         <v>1.1794616290406312</v>
       </c>
-      <c r="E7">
-        <f t="shared" si="4"/>
+      <c r="F8" s="5">
+        <f t="shared" si="5"/>
         <v>1.0920396561111183</v>
       </c>
-      <c r="F7">
+      <c r="G8" s="5">
+        <f t="shared" si="6"/>
+        <v>1.0447979842743009</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2017</v>
+      </c>
+      <c r="B9" s="5">
+        <v>254.738</v>
+      </c>
+      <c r="C9" s="5">
+        <f t="shared" si="2"/>
+        <v>1.3070095549152463</v>
+      </c>
+      <c r="D9" s="5">
+        <f t="shared" si="3"/>
+        <v>1.27124339517465</v>
+      </c>
+      <c r="E9" s="5">
+        <f t="shared" si="4"/>
+        <v>1.2189347486437045</v>
+      </c>
+      <c r="F9" s="5">
         <f t="shared" si="5"/>
-        <v>1.0447979842743009</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>2017</v>
-      </c>
-      <c r="B8" cm="1">
-        <f t="array" ref="B8">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A8,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>254.738</v>
-      </c>
-      <c r="C8">
-        <f t="shared" si="2"/>
-        <v>1.27124339517465</v>
-      </c>
-      <c r="D8">
-        <f t="shared" si="3"/>
-        <v>1.2189347486437045</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="4"/>
         <v>1.1285870188193361</v>
       </c>
-      <c r="F8">
+      <c r="G9" s="5">
+        <f t="shared" si="6"/>
+        <v>1.0797643068564564</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>2016</v>
+      </c>
+      <c r="B10" s="5">
+        <v>247.70500000000001</v>
+      </c>
+      <c r="C10" s="5">
+        <f t="shared" si="2"/>
+        <v>1.3441190125350719</v>
+      </c>
+      <c r="D10" s="5">
+        <f t="shared" si="3"/>
+        <v>1.3073373569366786</v>
+      </c>
+      <c r="E10" s="5">
+        <f t="shared" si="4"/>
+        <v>1.2535435296017441</v>
+      </c>
+      <c r="F10" s="5">
         <f t="shared" si="5"/>
-        <v>1.0797643068564564</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>2016</v>
-      </c>
-      <c r="B9" cm="1">
-        <f t="array" ref="B9">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A9,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>247.70500000000001</v>
-      </c>
-      <c r="C9">
-        <f t="shared" si="2"/>
-        <v>1.3073373569366786</v>
-      </c>
-      <c r="D9">
-        <f t="shared" si="3"/>
-        <v>1.2535435296017441</v>
-      </c>
-      <c r="E9">
-        <f t="shared" si="4"/>
         <v>1.1606305888052322</v>
       </c>
-      <c r="F9">
+      <c r="G10" s="5">
+        <f t="shared" si="6"/>
+        <v>1.1104216709392221</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>2015</v>
+      </c>
+      <c r="B11" s="5">
+        <v>243.01499999999999</v>
+      </c>
+      <c r="C11" s="5">
+        <f t="shared" si="2"/>
+        <v>1.3700594613501225</v>
+      </c>
+      <c r="D11" s="5">
+        <f t="shared" si="3"/>
+        <v>1.3325679484805466</v>
+      </c>
+      <c r="E11" s="5">
+        <f t="shared" si="4"/>
+        <v>1.2777359422257886</v>
+      </c>
+      <c r="F11" s="5">
         <f t="shared" si="5"/>
-        <v>1.1104216709392221</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>2015</v>
-      </c>
-      <c r="B10" cm="1">
-        <f t="array" ref="B10">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A10,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>243.01499999999999</v>
-      </c>
-      <c r="C10">
-        <f t="shared" si="2"/>
-        <v>1.3325679484805466</v>
-      </c>
-      <c r="D10">
-        <f t="shared" si="3"/>
-        <v>1.2777359422257886</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="4"/>
         <v>1.1830298541242312</v>
       </c>
-      <c r="F10">
+      <c r="G11" s="5">
+        <f t="shared" si="6"/>
+        <v>1.1318519432956815</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>2014</v>
+      </c>
+      <c r="B12" s="5">
+        <v>240.215</v>
+      </c>
+      <c r="C12" s="5">
+        <f t="shared" si="2"/>
+        <v>1.3860291821909538</v>
+      </c>
+      <c r="D12" s="5">
+        <f t="shared" si="3"/>
+        <v>1.3481006598255729</v>
+      </c>
+      <c r="E12" s="5">
+        <f t="shared" si="4"/>
+        <v>1.2926295193888808</v>
+      </c>
+      <c r="F12" s="5">
         <f t="shared" si="5"/>
-        <v>1.1318519432956815</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>2014</v>
-      </c>
-      <c r="B11" cm="1">
-        <f t="array" ref="B11">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A11,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>240.215</v>
-      </c>
-      <c r="C11">
-        <f t="shared" si="2"/>
-        <v>1.3481006598255729</v>
-      </c>
-      <c r="D11">
-        <f t="shared" si="3"/>
-        <v>1.2926295193888808</v>
-      </c>
-      <c r="E11">
-        <f t="shared" si="4"/>
         <v>1.196819515850384</v>
       </c>
-      <c r="F11">
+      <c r="G12" s="5">
+        <f t="shared" si="6"/>
+        <v>1.1450450637970153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>2013</v>
+      </c>
+      <c r="B13" s="5">
+        <v>235.82400000000001</v>
+      </c>
+      <c r="C13" s="5">
+        <f t="shared" si="2"/>
+        <v>1.4118367935409457</v>
+      </c>
+      <c r="D13" s="5">
+        <f t="shared" si="3"/>
+        <v>1.3732020489856842</v>
+      </c>
+      <c r="E13" s="5">
+        <f t="shared" si="4"/>
+        <v>1.3166980460004072</v>
+      </c>
+      <c r="F13" s="5">
         <f t="shared" si="5"/>
-        <v>1.1450450637970153</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>2013</v>
-      </c>
-      <c r="B12" cm="1">
-        <f t="array" ref="B12">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A12,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>235.82400000000001</v>
-      </c>
-      <c r="C12">
-        <f t="shared" si="2"/>
-        <v>1.3732020489856842</v>
-      </c>
-      <c r="D12">
-        <f t="shared" si="3"/>
-        <v>1.3166980460004072</v>
-      </c>
-      <c r="E12">
-        <f t="shared" si="4"/>
         <v>1.2191040776172062</v>
       </c>
-      <c r="F12">
+      <c r="G13" s="5">
+        <f t="shared" si="6"/>
+        <v>1.1663655946807789</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2012</v>
+      </c>
+      <c r="B14" s="5">
+        <v>232.376</v>
+      </c>
+      <c r="C14" s="5">
+        <f t="shared" si="2"/>
+        <v>1.4327856577271318</v>
+      </c>
+      <c r="D14" s="5">
+        <f t="shared" si="3"/>
+        <v>1.3935776500154922</v>
+      </c>
+      <c r="E14" s="5">
+        <f t="shared" si="4"/>
+        <v>1.3362352394395292</v>
+      </c>
+      <c r="F14" s="5">
         <f t="shared" si="5"/>
-        <v>1.1663655946807789</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>2012</v>
-      </c>
-      <c r="B13" cm="1">
-        <f t="array" ref="B13">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A13,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>232.376</v>
-      </c>
-      <c r="C13">
-        <f t="shared" si="2"/>
-        <v>1.3935776500154922</v>
-      </c>
-      <c r="D13">
-        <f t="shared" si="3"/>
-        <v>1.3362352394395292</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="4"/>
         <v>1.2371931696905016</v>
       </c>
-      <c r="F13">
+      <c r="G14" s="5">
+        <f t="shared" si="6"/>
+        <v>1.1836721520294695</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2011</v>
+      </c>
+      <c r="B15" s="5">
+        <v>227.48500000000001</v>
+      </c>
+      <c r="C15" s="5">
+        <f t="shared" si="2"/>
+        <v>1.4635910060003956</v>
+      </c>
+      <c r="D15" s="5">
+        <f t="shared" si="3"/>
+        <v>1.423540013627272</v>
+      </c>
+      <c r="E15" s="5">
+        <f t="shared" si="4"/>
+        <v>1.3649647229487658</v>
+      </c>
+      <c r="F15" s="5">
         <f t="shared" si="5"/>
-        <v>1.1836721520294695</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>2011</v>
-      </c>
-      <c r="B14" cm="1">
-        <f t="array" ref="B14">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A14,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>227.48500000000001</v>
-      </c>
-      <c r="C14">
-        <f t="shared" si="2"/>
-        <v>1.423540013627272</v>
-      </c>
-      <c r="D14">
-        <f t="shared" si="3"/>
-        <v>1.3649647229487658</v>
-      </c>
-      <c r="E14">
-        <f t="shared" si="4"/>
         <v>1.2637932171351958</v>
       </c>
-      <c r="F14">
+      <c r="G15" s="5">
+        <f t="shared" si="6"/>
+        <v>1.2091214805371784</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2010</v>
+      </c>
+      <c r="B16" s="5">
+        <v>221.203</v>
+      </c>
+      <c r="C16" s="5">
+        <f t="shared" si="2"/>
+        <v>1.5051558975239938</v>
+      </c>
+      <c r="D16" s="5">
+        <f t="shared" si="3"/>
+        <v>1.4639674868785686</v>
+      </c>
+      <c r="E16" s="5">
+        <f t="shared" si="4"/>
+        <v>1.4037287016903026</v>
+      </c>
+      <c r="F16" s="5">
         <f t="shared" si="5"/>
-        <v>1.2091214805371784</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>2010</v>
-      </c>
-      <c r="B15" cm="1">
-        <f t="array" ref="B15">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A15,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>221.203</v>
-      </c>
-      <c r="C15">
-        <f t="shared" si="2"/>
-        <v>1.4639674868785686</v>
-      </c>
-      <c r="D15">
-        <f t="shared" si="3"/>
-        <v>1.4037287016903026</v>
-      </c>
-      <c r="E15">
-        <f t="shared" si="4"/>
         <v>1.2996840006690689</v>
       </c>
-      <c r="F15">
+      <c r="G16" s="5">
+        <f t="shared" si="6"/>
+        <v>1.2434596275819045</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2009</v>
+      </c>
+      <c r="B17" s="5">
+        <v>218.822</v>
+      </c>
+      <c r="C17" s="5">
+        <f t="shared" si="2"/>
+        <v>1.5215334838361774</v>
+      </c>
+      <c r="D17" s="5">
+        <f t="shared" si="3"/>
+        <v>1.4798969025052326</v>
+      </c>
+      <c r="E17" s="5">
+        <f t="shared" si="4"/>
+        <v>1.4190026596960086</v>
+      </c>
+      <c r="F17" s="5">
         <f t="shared" si="5"/>
-        <v>1.2434596275819045</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>2009</v>
-      </c>
-      <c r="B16" cm="1">
-        <f t="array" ref="B16">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A16,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>218.822</v>
-      </c>
-      <c r="C16">
-        <f t="shared" si="2"/>
-        <v>1.4798969025052326</v>
-      </c>
-      <c r="D16">
-        <f t="shared" si="3"/>
-        <v>1.4190026596960086</v>
-      </c>
-      <c r="E16">
-        <f t="shared" si="4"/>
         <v>1.3138258493204524</v>
       </c>
-      <c r="F16">
+      <c r="G17" s="5">
+        <f t="shared" si="6"/>
+        <v>1.2569896993903722</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2008</v>
+      </c>
+      <c r="B18" s="5">
+        <v>219.64599999999999</v>
+      </c>
+      <c r="C18" s="5">
+        <f t="shared" si="2"/>
+        <v>1.5158254646112381</v>
+      </c>
+      <c r="D18" s="5">
+        <f t="shared" si="3"/>
+        <v>1.4743450825419084</v>
+      </c>
+      <c r="E18" s="5">
+        <f t="shared" si="4"/>
+        <v>1.4136792839387016</v>
+      </c>
+      <c r="F18" s="5">
         <f t="shared" si="5"/>
-        <v>1.2569896993903722</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>2008</v>
-      </c>
-      <c r="B17" cm="1">
-        <f t="array" ref="B17">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A17,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>219.64599999999999</v>
-      </c>
-      <c r="C17">
-        <f t="shared" si="2"/>
-        <v>1.4743450825419084</v>
-      </c>
-      <c r="D17">
-        <f t="shared" si="3"/>
-        <v>1.4136792839387016</v>
-      </c>
-      <c r="E17">
-        <f t="shared" si="4"/>
         <v>1.3088970434244196</v>
       </c>
-      <c r="F17">
+      <c r="G18" s="5">
+        <f t="shared" si="6"/>
+        <v>1.2522741138012985</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2007</v>
+      </c>
+      <c r="B19" s="5">
+        <v>212.23</v>
+      </c>
+      <c r="C19" s="5">
+        <f t="shared" si="2"/>
+        <v>1.5687932902982613</v>
+      </c>
+      <c r="D19" s="5">
+        <f t="shared" si="3"/>
+        <v>1.5258634500306272</v>
+      </c>
+      <c r="E19" s="5">
+        <f t="shared" si="4"/>
+        <v>1.4630777929604675</v>
+      </c>
+      <c r="F19" s="5">
         <f t="shared" si="5"/>
-        <v>1.2522741138012985</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>2007</v>
-      </c>
-      <c r="B18" cm="1">
-        <f t="array" ref="B18">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A18,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>212.23</v>
-      </c>
-      <c r="C18">
-        <f t="shared" si="2"/>
-        <v>1.5258634500306272</v>
-      </c>
-      <c r="D18">
-        <f t="shared" si="3"/>
-        <v>1.4630777929604675</v>
-      </c>
-      <c r="E18">
-        <f t="shared" si="4"/>
         <v>1.3546341233567358</v>
       </c>
-      <c r="F18">
+      <c r="G19" s="5">
+        <f t="shared" si="6"/>
+        <v>1.2960326061348539</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2006</v>
+      </c>
+      <c r="B20" s="5">
+        <v>205.7</v>
+      </c>
+      <c r="C20" s="5">
+        <f t="shared" si="2"/>
+        <v>1.618595041322314</v>
+      </c>
+      <c r="D20" s="5">
+        <f t="shared" si="3"/>
+        <v>1.5743023821098689</v>
+      </c>
+      <c r="E20" s="5">
+        <f t="shared" si="4"/>
+        <v>1.5095235780262519</v>
+      </c>
+      <c r="F20" s="5">
         <f t="shared" si="5"/>
-        <v>1.2960326061348539</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>2006</v>
-      </c>
-      <c r="B19" cm="1">
-        <f t="array" ref="B19">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A19,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>205.7</v>
-      </c>
-      <c r="C19">
-        <f t="shared" si="2"/>
-        <v>1.5743023821098689</v>
-      </c>
-      <c r="D19">
-        <f t="shared" si="3"/>
-        <v>1.5095235780262519</v>
-      </c>
-      <c r="E19">
-        <f t="shared" si="4"/>
         <v>1.3976373359261063</v>
       </c>
-      <c r="F19">
+      <c r="G20" s="5">
+        <f t="shared" si="6"/>
+        <v>1.3371754982984931</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>2005</v>
+      </c>
+      <c r="B21" s="5">
+        <v>198.9</v>
+      </c>
+      <c r="C21" s="5">
+        <f t="shared" si="2"/>
+        <v>1.6739316239316238</v>
+      </c>
+      <c r="D21" s="5">
+        <f t="shared" si="3"/>
+        <v>1.6281246857717446</v>
+      </c>
+      <c r="E21" s="5">
+        <f t="shared" si="4"/>
+        <v>1.5611312217194571</v>
+      </c>
+      <c r="F21" s="5">
         <f t="shared" si="5"/>
-        <v>1.3371754982984931</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>2005</v>
-      </c>
-      <c r="B20" cm="1">
-        <f t="array" ref="B20">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A20,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>198.9</v>
-      </c>
-      <c r="C20">
-        <f t="shared" si="2"/>
-        <v>1.6281246857717446</v>
-      </c>
-      <c r="D20">
-        <f t="shared" si="3"/>
-        <v>1.5611312217194571</v>
-      </c>
-      <c r="E20">
-        <f t="shared" si="4"/>
         <v>1.4454198089492207</v>
       </c>
-      <c r="F20">
+      <c r="G21" s="5">
+        <f t="shared" si="6"/>
+        <v>1.3828908999497236</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2004</v>
+      </c>
+      <c r="B22" s="5">
+        <v>193</v>
+      </c>
+      <c r="C22" s="5">
+        <f t="shared" si="2"/>
+        <v>1.7251036269430051</v>
+      </c>
+      <c r="D22" s="5">
+        <f t="shared" si="3"/>
+        <v>1.6778963730569949</v>
+      </c>
+      <c r="E22" s="5">
+        <f t="shared" si="4"/>
+        <v>1.6088549222797928</v>
+      </c>
+      <c r="F22" s="5">
         <f t="shared" si="5"/>
-        <v>1.3828908999497236</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>2004</v>
-      </c>
-      <c r="B21" cm="1">
-        <f t="array" ref="B21">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A21,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>193</v>
-      </c>
-      <c r="C21">
-        <f t="shared" si="2"/>
-        <v>1.6778963730569949</v>
-      </c>
-      <c r="D21">
-        <f t="shared" si="3"/>
-        <v>1.6088549222797928</v>
-      </c>
-      <c r="E21">
-        <f t="shared" si="4"/>
         <v>1.4896062176165805</v>
       </c>
-      <c r="F21">
+      <c r="G22" s="5">
+        <f t="shared" si="6"/>
+        <v>1.4251658031088084</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2003</v>
+      </c>
+      <c r="B23" s="5">
+        <v>188.6</v>
+      </c>
+      <c r="C23" s="5">
+        <f t="shared" si="2"/>
+        <v>1.7653499469777307</v>
+      </c>
+      <c r="D23" s="5">
+        <f t="shared" si="3"/>
+        <v>1.7170413573700956</v>
+      </c>
+      <c r="E23" s="5">
+        <f t="shared" si="4"/>
+        <v>1.6463891834570521</v>
+      </c>
+      <c r="F23" s="5">
         <f t="shared" si="5"/>
-        <v>1.4251658031088084</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>2003</v>
-      </c>
-      <c r="B22" cm="1">
-        <f t="array" ref="B22">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A22,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>188.6</v>
-      </c>
-      <c r="C22">
-        <f t="shared" si="2"/>
-        <v>1.7170413573700956</v>
-      </c>
-      <c r="D22">
-        <f t="shared" si="3"/>
-        <v>1.6463891834570521</v>
-      </c>
-      <c r="E22">
-        <f t="shared" si="4"/>
         <v>1.5243584305408273</v>
       </c>
-      <c r="F22">
+      <c r="G23" s="5">
+        <f t="shared" si="6"/>
+        <v>1.4584146341463415</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2002</v>
+      </c>
+      <c r="B24" s="5">
+        <v>184.7</v>
+      </c>
+      <c r="C24" s="5">
+        <f t="shared" si="2"/>
+        <v>1.8026258798050894</v>
+      </c>
+      <c r="D24" s="5">
+        <f t="shared" si="3"/>
+        <v>1.7532972387655659</v>
+      </c>
+      <c r="E24" s="5">
+        <f t="shared" si="4"/>
+        <v>1.6811532214401734</v>
+      </c>
+      <c r="F24" s="5">
         <f t="shared" si="5"/>
-        <v>1.4584146341463415</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>2002</v>
-      </c>
-      <c r="B23" cm="1">
-        <f t="array" ref="B23">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A23,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>184.7</v>
-      </c>
-      <c r="C23">
-        <f t="shared" si="2"/>
-        <v>1.7532972387655659</v>
-      </c>
-      <c r="D23">
-        <f t="shared" si="3"/>
-        <v>1.6811532214401734</v>
-      </c>
-      <c r="E23">
-        <f t="shared" si="4"/>
         <v>1.5565457498646456</v>
       </c>
-      <c r="F23">
+      <c r="G24" s="5">
+        <f t="shared" si="6"/>
+        <v>1.4892095289658909</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2001</v>
+      </c>
+      <c r="B25" s="5">
+        <v>181.2</v>
+      </c>
+      <c r="C25" s="5">
+        <f t="shared" si="2"/>
+        <v>1.8374448123620311</v>
+      </c>
+      <c r="D25" s="5">
+        <f t="shared" si="3"/>
+        <v>1.7871633554083886</v>
+      </c>
+      <c r="E25" s="5">
+        <f t="shared" si="4"/>
+        <v>1.7136258278145697</v>
+      </c>
+      <c r="F25" s="5">
         <f t="shared" si="5"/>
-        <v>1.4892095289658909</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>2001</v>
-      </c>
-      <c r="B24" cm="1">
-        <f t="array" ref="B24">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A24,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>181.2</v>
-      </c>
-      <c r="C24">
-        <f t="shared" si="2"/>
-        <v>1.7871633554083886</v>
-      </c>
-      <c r="D24">
-        <f t="shared" si="3"/>
-        <v>1.7136258278145697</v>
-      </c>
-      <c r="E24">
-        <f t="shared" si="4"/>
         <v>1.5866114790286978</v>
       </c>
-      <c r="F24">
+      <c r="G25" s="5">
+        <f t="shared" si="6"/>
+        <v>1.5179746136865344</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2000</v>
+      </c>
+      <c r="B26" s="5">
+        <v>174.8</v>
+      </c>
+      <c r="C26" s="5">
+        <f t="shared" si="2"/>
+        <v>1.904719679633867</v>
+      </c>
+      <c r="D26" s="5">
+        <f t="shared" si="3"/>
+        <v>1.8525972540045765</v>
+      </c>
+      <c r="E26" s="5">
+        <f t="shared" si="4"/>
+        <v>1.7763672768878718</v>
+      </c>
+      <c r="F26" s="5">
         <f t="shared" si="5"/>
-        <v>1.5179746136865344</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>2000</v>
-      </c>
-      <c r="B25" cm="1">
-        <f t="array" ref="B25">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A25,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>174.8</v>
-      </c>
-      <c r="C25">
-        <f t="shared" si="2"/>
-        <v>1.8525972540045765</v>
-      </c>
-      <c r="D25">
-        <f t="shared" si="3"/>
-        <v>1.7763672768878718</v>
-      </c>
-      <c r="E25">
-        <f t="shared" si="4"/>
         <v>1.6447025171624714</v>
       </c>
-      <c r="F25">
+      <c r="G26" s="5">
+        <f t="shared" si="6"/>
+        <v>1.5735526315789474</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>1999</v>
+      </c>
+      <c r="B27" s="5">
+        <v>168.9</v>
+      </c>
+      <c r="C27" s="5">
+        <f t="shared" si="2"/>
+        <v>1.971255180580225</v>
+      </c>
+      <c r="D27" s="5">
+        <f t="shared" si="3"/>
+        <v>1.9173120189461219</v>
+      </c>
+      <c r="E27" s="5">
+        <f t="shared" si="4"/>
+        <v>1.8384191829484902</v>
+      </c>
+      <c r="F27" s="5">
         <f t="shared" si="5"/>
-        <v>1.5735526315789474</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>1999</v>
-      </c>
-      <c r="B26" cm="1">
-        <f t="array" ref="B26">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A26,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>168.9</v>
-      </c>
-      <c r="C26">
-        <f t="shared" si="2"/>
-        <v>1.9173120189461219</v>
-      </c>
-      <c r="D26">
-        <f t="shared" si="3"/>
-        <v>1.8384191829484902</v>
-      </c>
-      <c r="E26">
-        <f t="shared" si="4"/>
         <v>1.7021551213735939</v>
       </c>
-      <c r="F26">
+      <c r="G27" s="5">
+        <f t="shared" si="6"/>
+        <v>1.6285198342214329</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>1998</v>
+      </c>
+      <c r="B28" s="5">
+        <v>164.4</v>
+      </c>
+      <c r="C28" s="5">
+        <f t="shared" si="2"/>
+        <v>2.0252128953771287</v>
+      </c>
+      <c r="D28" s="5">
+        <f t="shared" si="3"/>
+        <v>1.9697931873479317</v>
+      </c>
+      <c r="E28" s="5">
+        <f t="shared" si="4"/>
+        <v>1.8887408759124087</v>
+      </c>
+      <c r="F28" s="5">
         <f t="shared" si="5"/>
-        <v>1.6285198342214329</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>1998</v>
-      </c>
-      <c r="B27" cm="1">
-        <f t="array" ref="B27">INDEX('[1]monthly cpi west'!R$12:R$37, MATCH(A27,'[1]monthly cpi west'!E$12:E$38, 0), 0)</f>
-        <v>164.4</v>
-      </c>
-      <c r="C27">
-        <f t="shared" si="2"/>
-        <v>1.9697931873479317</v>
-      </c>
-      <c r="D27">
-        <f t="shared" si="3"/>
-        <v>1.8887408759124087</v>
-      </c>
-      <c r="E27">
-        <f t="shared" si="4"/>
         <v>1.7487469586374698</v>
       </c>
-      <c r="F27">
-        <f t="shared" si="5"/>
+      <c r="G28" s="5">
+        <f t="shared" si="6"/>
         <v>1.6730961070559611</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Formatting updates all around
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/CPI_IAF.xlsx
+++ b/Indicator_Gen/config/CPI_IAF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7901D95-8F4E-4CAE-A549-BFDC9647AB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{283EAA62-5D11-410D-A9F3-18618E38D914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="7" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="322">
   <si>
     <t>Year</t>
   </si>
@@ -1436,15 +1436,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A1D1C33-6ADD-4F8E-BC64-E68634ED55EB}">
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:O71"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.59765625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="11.8984375" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="14" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.8984375" style="5" customWidth="1"/>
+    <col min="4" max="7" width="11.8984375" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="15" width="11.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1452,18 +1453,20 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -1471,1660 +1474,1965 @@
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B2" s="5">
-        <v>331.80399999999997</v>
+        <v>341.95100000000002</v>
       </c>
       <c r="C2" s="5">
-        <f t="shared" ref="C2:C33" si="0">$B$2/B2</f>
+        <f t="shared" ref="C2:C67" si="0">$B$2/B2</f>
         <v>1</v>
       </c>
       <c r="D2" s="5">
-        <f>$B$3/B2</f>
-        <v>0.96208605080107534</v>
+        <f t="shared" ref="D2:D34" si="1">$B$3/B2</f>
+        <v>0.97032615784132803</v>
       </c>
       <c r="E2" s="5">
         <f>$B$4/B2</f>
-        <v>0.89622487974828513</v>
+        <v>0.93353726118654423</v>
       </c>
       <c r="F2" s="5">
         <f>$B$5/B2</f>
-        <v>0.85989017612807572</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0.86963044412795976</v>
+      </c>
+      <c r="G2" s="5">
+        <f>$B$6/B2</f>
+        <v>0.83437393076785848</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B3" s="5">
-        <v>319.22399999999999</v>
+        <v>331.80399999999997</v>
       </c>
       <c r="C3" s="5">
         <f t="shared" si="0"/>
-        <v>1.0394080645565495</v>
+        <v>1.0305813070366845</v>
       </c>
       <c r="D3" s="5">
-        <f t="shared" ref="D3:D66" si="1">$B$3/B3</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E3" s="5">
-        <f t="shared" ref="E3:E66" si="2">$B$4/B3</f>
-        <v>0.9315433676665914</v>
+        <f>$B$4/B3</f>
+        <v>0.96208605080107534</v>
       </c>
       <c r="F3" s="5">
-        <f t="shared" ref="F3:F66" si="3">$B$5/B3</f>
-        <v>0.89377678370047364</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <f>$B$5/B3</f>
+        <v>0.89622487974828513</v>
+      </c>
+      <c r="G3" s="5">
+        <f>$B$6/B3</f>
+        <v>0.85989017612807572</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B4" s="5">
-        <v>297.37099999999998</v>
+        <v>319.22399999999999</v>
       </c>
       <c r="C4" s="5">
         <f t="shared" si="0"/>
-        <v>1.1157913851720578</v>
+        <v>1.0711945217151593</v>
       </c>
       <c r="D4" s="5">
         <f t="shared" si="1"/>
-        <v>1.0734873272780467</v>
+        <v>1.0394080645565495</v>
       </c>
       <c r="E4" s="5">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="E4:E67" si="2">$B$4/B4</f>
         <v>1</v>
       </c>
       <c r="F4" s="5">
-        <f t="shared" si="3"/>
-        <v>0.95945805071779033</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="shared" ref="F4:F67" si="3">$B$5/B4</f>
+        <v>0.9315433676665914</v>
+      </c>
+      <c r="G4" s="5">
+        <f t="shared" ref="G4:G67" si="4">$B$6/B4</f>
+        <v>0.89377678370047364</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B5" s="5">
-        <v>285.315</v>
+        <v>297.37099999999998</v>
       </c>
       <c r="C5" s="5">
         <f t="shared" si="0"/>
-        <v>1.1629392075425407</v>
+        <v>1.149913744110892</v>
       </c>
       <c r="D5" s="5">
         <f t="shared" si="1"/>
-        <v>1.118847589506335</v>
+        <v>1.1157913851720578</v>
       </c>
       <c r="E5" s="5">
         <f t="shared" si="2"/>
-        <v>1.0422550514343796</v>
+        <v>1.0734873272780467</v>
       </c>
       <c r="F5" s="5">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G5" s="5">
+        <f t="shared" si="4"/>
+        <v>0.95945805071779033</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B6" s="5">
-        <v>280.63799999999998</v>
+        <v>285.315</v>
       </c>
       <c r="C6" s="5">
         <f t="shared" si="0"/>
-        <v>1.1823202844946159</v>
+        <v>1.1985034085133977</v>
       </c>
       <c r="D6" s="5">
         <f t="shared" si="1"/>
-        <v>1.1374938532914289</v>
+        <v>1.1629392075425407</v>
       </c>
       <c r="E6" s="5">
         <f t="shared" si="2"/>
-        <v>1.0596248547951455</v>
+        <v>1.118847589506335</v>
       </c>
       <c r="F6" s="5">
         <f t="shared" si="3"/>
-        <v>1.0166655976738717</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.0422550514343796</v>
+      </c>
+      <c r="G6" s="5">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B7" s="5">
-        <v>272.51</v>
+        <v>280.63799999999998</v>
       </c>
       <c r="C7" s="5">
         <f t="shared" si="0"/>
-        <v>1.2175846757917139</v>
+        <v>1.2184771841304458</v>
       </c>
       <c r="D7" s="5">
         <f t="shared" si="1"/>
-        <v>1.1714212322483579</v>
+        <v>1.1823202844946159</v>
       </c>
       <c r="E7" s="5">
         <f t="shared" si="2"/>
-        <v>1.0912296796447836</v>
+        <v>1.1374938532914289</v>
       </c>
       <c r="F7" s="5">
         <f t="shared" si="3"/>
-        <v>1.0469891013173829</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.0596248547951455</v>
+      </c>
+      <c r="G7" s="5">
+        <f t="shared" si="4"/>
+        <v>1.0166655976738717</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B8" s="5">
-        <v>262.80200000000002</v>
+        <v>272.51</v>
       </c>
       <c r="C8" s="5">
         <f t="shared" si="0"/>
-        <v>1.2625626897816604</v>
+        <v>1.2548200066052624</v>
       </c>
       <c r="D8" s="5">
         <f t="shared" si="1"/>
-        <v>1.2146939521008211</v>
+        <v>1.2175846757917139</v>
       </c>
       <c r="E8" s="5">
         <f t="shared" si="2"/>
-        <v>1.1315400948242402</v>
+        <v>1.1714212322483579</v>
       </c>
       <c r="F8" s="5">
         <f t="shared" si="3"/>
-        <v>1.0856652536890889</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.0912296796447836</v>
+      </c>
+      <c r="G8" s="5">
+        <f t="shared" si="4"/>
+        <v>1.0469891013173829</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="B9" s="5">
-        <v>255.303</v>
+        <v>262.80200000000002</v>
       </c>
       <c r="C9" s="5">
         <f t="shared" si="0"/>
-        <v>1.2996478693944058</v>
+        <v>1.3011735070509356</v>
       </c>
       <c r="D9" s="5">
         <f t="shared" si="1"/>
-        <v>1.2503730860976956</v>
+        <v>1.2625626897816604</v>
       </c>
       <c r="E9" s="5">
         <f t="shared" si="2"/>
-        <v>1.1647767554631163</v>
+        <v>1.2146939521008211</v>
       </c>
       <c r="F9" s="5">
         <f t="shared" si="3"/>
-        <v>1.1175544353180338</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.1315400948242402</v>
+      </c>
+      <c r="G9" s="5">
+        <f t="shared" si="4"/>
+        <v>1.0856652536890889</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="B10" s="5">
-        <v>249.666</v>
+        <v>255.303</v>
       </c>
       <c r="C10" s="5">
         <f t="shared" si="0"/>
-        <v>1.3289915326876707</v>
+        <v>1.3393927999279289</v>
       </c>
       <c r="D10" s="5">
         <f t="shared" si="1"/>
-        <v>1.2786042152315493</v>
+        <v>1.2996478693944058</v>
       </c>
       <c r="E10" s="5">
         <f t="shared" si="2"/>
-        <v>1.1910752765694967</v>
+        <v>1.2503730860976956</v>
       </c>
       <c r="F10" s="5">
         <f t="shared" si="3"/>
-        <v>1.1427867631155224</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.1647767554631163</v>
+      </c>
+      <c r="G10" s="5">
+        <f t="shared" si="4"/>
+        <v>1.1175544353180338</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="B11" s="5">
-        <v>246.05500000000001</v>
+        <v>249.666</v>
       </c>
       <c r="C11" s="5">
         <f t="shared" si="0"/>
-        <v>1.3484952551258864</v>
+        <v>1.3696338307979461</v>
       </c>
       <c r="D11" s="5">
         <f t="shared" si="1"/>
-        <v>1.2973684745280525</v>
+        <v>1.3289915326876707</v>
       </c>
       <c r="E11" s="5">
         <f t="shared" si="2"/>
-        <v>1.2085549978663306</v>
+        <v>1.2786042152315493</v>
       </c>
       <c r="F11" s="5">
         <f t="shared" si="3"/>
-        <v>1.1595578224380727</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.1910752765694967</v>
+      </c>
+      <c r="G11" s="5">
+        <f t="shared" si="4"/>
+        <v>1.1427867631155224</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="B12" s="5">
-        <v>241.62299999999999</v>
+        <v>246.05500000000001</v>
       </c>
       <c r="C12" s="5">
         <f t="shared" si="0"/>
-        <v>1.3732301974563679</v>
+        <v>1.3897340025604032</v>
       </c>
       <c r="D12" s="5">
         <f t="shared" si="1"/>
-        <v>1.321165617511578</v>
+        <v>1.3484952551258864</v>
       </c>
       <c r="E12" s="5">
         <f t="shared" si="2"/>
-        <v>1.2307230685820472</v>
+        <v>1.2973684745280525</v>
       </c>
       <c r="F12" s="5">
         <f t="shared" si="3"/>
-        <v>1.1808271563551485</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.2085549978663306</v>
+      </c>
+      <c r="G12" s="5">
+        <f t="shared" si="4"/>
+        <v>1.1595578224380727</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="B13" s="5">
-        <v>238.155</v>
+        <v>241.62299999999999</v>
       </c>
       <c r="C13" s="5">
         <f t="shared" si="0"/>
-        <v>1.3932270999979004</v>
+        <v>1.4152253717568279</v>
       </c>
       <c r="D13" s="5">
         <f t="shared" si="1"/>
-        <v>1.340404358506015</v>
+        <v>1.3732301974563679</v>
       </c>
       <c r="E13" s="5">
         <f t="shared" si="2"/>
-        <v>1.2486447901576703</v>
+        <v>1.321165617511578</v>
       </c>
       <c r="F13" s="5">
         <f t="shared" si="3"/>
-        <v>1.1980222964036027</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.2307230685820472</v>
+      </c>
+      <c r="G13" s="5">
+        <f t="shared" si="4"/>
+        <v>1.1808271563551485</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="B14" s="5">
-        <v>232.93</v>
+        <v>238.155</v>
       </c>
       <c r="C14" s="5">
         <f t="shared" si="0"/>
-        <v>1.4244794573477009</v>
+        <v>1.4358338057147657</v>
       </c>
       <c r="D14" s="5">
         <f t="shared" si="1"/>
-        <v>1.3704718155669084</v>
+        <v>1.3932270999979004</v>
       </c>
       <c r="E14" s="5">
         <f t="shared" si="2"/>
-        <v>1.2766539303653457</v>
+        <v>1.340404358506015</v>
       </c>
       <c r="F14" s="5">
         <f t="shared" si="3"/>
-        <v>1.2248958914695403</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.2486447901576703</v>
+      </c>
+      <c r="G14" s="5">
+        <f t="shared" si="4"/>
+        <v>1.1980222964036027</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="B15" s="5">
-        <v>226.91900000000001</v>
+        <v>232.93</v>
       </c>
       <c r="C15" s="5">
         <f t="shared" si="0"/>
-        <v>1.4622133889185125</v>
+        <v>1.4680419010003005</v>
       </c>
       <c r="D15" s="5">
         <f t="shared" si="1"/>
-        <v>1.4067751047730688</v>
+        <v>1.4244794573477009</v>
       </c>
       <c r="E15" s="5">
         <f t="shared" si="2"/>
-        <v>1.3104720186498264</v>
+        <v>1.3704718155669084</v>
       </c>
       <c r="F15" s="5">
         <f t="shared" si="3"/>
-        <v>1.2573429285339701</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+        <v>1.2766539303653457</v>
+      </c>
+      <c r="G15" s="5">
+        <f t="shared" si="4"/>
+        <v>1.2248958914695403</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="B16" s="5">
-        <v>224.11</v>
+        <v>226.91900000000001</v>
       </c>
       <c r="C16" s="5">
         <f t="shared" si="0"/>
-        <v>1.4805408058542677</v>
+        <v>1.5069297855181805</v>
       </c>
       <c r="D16" s="5">
         <f t="shared" si="1"/>
-        <v>1.4244076569541742</v>
+        <v>1.4622133889185125</v>
       </c>
       <c r="E16" s="5">
         <f t="shared" si="2"/>
-        <v>1.3268975056891703</v>
+        <v>1.4067751047730688</v>
       </c>
       <c r="F16" s="5">
         <f t="shared" si="3"/>
-        <v>1.2731024943108293</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.3104720186498264</v>
+      </c>
+      <c r="G16" s="5">
+        <f t="shared" si="4"/>
+        <v>1.2573429285339701</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="B17" s="5">
-        <v>224.80699999999999</v>
+        <v>224.11</v>
       </c>
       <c r="C17" s="5">
         <f t="shared" si="0"/>
-        <v>1.4759504819689777</v>
+        <v>1.5258176788184374</v>
       </c>
       <c r="D17" s="5">
         <f t="shared" si="1"/>
-        <v>1.4199913703754776</v>
+        <v>1.4805408058542677</v>
       </c>
       <c r="E17" s="5">
         <f t="shared" si="2"/>
-        <v>1.3227835432170707</v>
+        <v>1.4244076569541742</v>
       </c>
       <c r="F17" s="5">
         <f t="shared" si="3"/>
-        <v>1.2691553198966226</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.3268975056891703</v>
+      </c>
+      <c r="G17" s="5">
+        <f t="shared" si="4"/>
+        <v>1.2731024943108293</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="B18" s="5">
-        <v>217.42400000000001</v>
+        <v>224.80699999999999</v>
       </c>
       <c r="C18" s="5">
         <f t="shared" si="0"/>
-        <v>1.5260688792405621</v>
+        <v>1.5210869768290136</v>
       </c>
       <c r="D18" s="5">
         <f t="shared" si="1"/>
-        <v>1.4682095812789755</v>
+        <v>1.4759504819689777</v>
       </c>
       <c r="E18" s="5">
         <f t="shared" si="2"/>
-        <v>1.3677008977849729</v>
+        <v>1.4199913703754776</v>
       </c>
       <c r="F18" s="5">
         <f t="shared" si="3"/>
-        <v>1.3122516373537418</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.3227835432170707</v>
+      </c>
+      <c r="G18" s="5">
+        <f t="shared" si="4"/>
+        <v>1.2691553198966226</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="B19" s="5">
-        <v>210.5</v>
+        <v>217.42400000000001</v>
       </c>
       <c r="C19" s="5">
         <f t="shared" si="0"/>
-        <v>1.5762660332541567</v>
+        <v>1.5727380601957466</v>
       </c>
       <c r="D19" s="5">
         <f t="shared" si="1"/>
-        <v>1.516503562945368</v>
+        <v>1.5260688792405621</v>
       </c>
       <c r="E19" s="5">
         <f t="shared" si="2"/>
-        <v>1.4126888361045129</v>
+        <v>1.4682095812789755</v>
       </c>
       <c r="F19" s="5">
         <f t="shared" si="3"/>
-        <v>1.35541567695962</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.3677008977849729</v>
+      </c>
+      <c r="G19" s="5">
+        <f t="shared" si="4"/>
+        <v>1.3122516373537418</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="B20" s="5">
-        <v>202.6</v>
+        <v>210.5</v>
       </c>
       <c r="C20" s="5">
         <f t="shared" si="0"/>
-        <v>1.6377295162882526</v>
+        <v>1.6244703087885988</v>
       </c>
       <c r="D20" s="5">
         <f t="shared" si="1"/>
-        <v>1.5756367226061205</v>
+        <v>1.5762660332541567</v>
       </c>
       <c r="E20" s="5">
         <f t="shared" si="2"/>
-        <v>1.4677739387956563</v>
+        <v>1.516503562945368</v>
       </c>
       <c r="F20" s="5">
         <f t="shared" si="3"/>
-        <v>1.4082675222112537</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.4126888361045129</v>
+      </c>
+      <c r="G20" s="5">
+        <f t="shared" si="4"/>
+        <v>1.35541567695962</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="B21" s="5">
-        <v>195.4</v>
+        <v>202.6</v>
       </c>
       <c r="C21" s="5">
         <f t="shared" si="0"/>
-        <v>1.6980757420675536</v>
+        <v>1.6878134254689043</v>
       </c>
       <c r="D21" s="5">
         <f t="shared" si="1"/>
-        <v>1.633694984646878</v>
+        <v>1.6377295162882526</v>
       </c>
       <c r="E21" s="5">
         <f t="shared" si="2"/>
-        <v>1.5218577277379732</v>
+        <v>1.5756367226061205</v>
       </c>
       <c r="F21" s="5">
         <f t="shared" si="3"/>
-        <v>1.4601586489252814</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.4677739387956563</v>
+      </c>
+      <c r="G21" s="5">
+        <f t="shared" si="4"/>
+        <v>1.4082675222112537</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="B22" s="5">
-        <v>190.4</v>
+        <v>195.4</v>
       </c>
       <c r="C22" s="5">
         <f t="shared" si="0"/>
-        <v>1.7426680672268906</v>
+        <v>1.7500051177072673</v>
       </c>
       <c r="D22" s="5">
         <f t="shared" si="1"/>
-        <v>1.676596638655462</v>
+        <v>1.6980757420675536</v>
       </c>
       <c r="E22" s="5">
         <f t="shared" si="2"/>
-        <v>1.5618224789915964</v>
+        <v>1.633694984646878</v>
       </c>
       <c r="F22" s="5">
         <f t="shared" si="3"/>
-        <v>1.498503151260504</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.5218577277379732</v>
+      </c>
+      <c r="G22" s="5">
+        <f t="shared" si="4"/>
+        <v>1.4601586489252814</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="B23" s="5">
-        <v>186.1</v>
+        <v>190.4</v>
       </c>
       <c r="C23" s="5">
         <f t="shared" si="0"/>
-        <v>1.7829339065018805</v>
+        <v>1.7959611344537816</v>
       </c>
       <c r="D23" s="5">
         <f t="shared" si="1"/>
-        <v>1.715335840945728</v>
+        <v>1.7426680672268906</v>
       </c>
       <c r="E23" s="5">
         <f t="shared" si="2"/>
-        <v>1.5979097259537882</v>
+        <v>1.676596638655462</v>
       </c>
       <c r="F23" s="5">
         <f t="shared" si="3"/>
-        <v>1.5331273508866201</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.5618224789915964</v>
+      </c>
+      <c r="G23" s="5">
+        <f t="shared" si="4"/>
+        <v>1.498503151260504</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="B24" s="5">
-        <v>181.7</v>
+        <v>186.1</v>
       </c>
       <c r="C24" s="5">
         <f t="shared" si="0"/>
-        <v>1.8261089708310401</v>
+        <v>1.83745835572273</v>
       </c>
       <c r="D24" s="5">
         <f t="shared" si="1"/>
-        <v>1.7568739680792516</v>
+        <v>1.7829339065018805</v>
       </c>
       <c r="E24" s="5">
         <f t="shared" si="2"/>
-        <v>1.6366042927903137</v>
+        <v>1.715335840945728</v>
       </c>
       <c r="F24" s="5">
         <f t="shared" si="3"/>
-        <v>1.5702531645569622</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.5979097259537882</v>
+      </c>
+      <c r="G24" s="5">
+        <f t="shared" si="4"/>
+        <v>1.5331273508866201</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="B25" s="5">
-        <v>174.8</v>
+        <v>181.7</v>
       </c>
       <c r="C25" s="5">
         <f t="shared" si="0"/>
-        <v>1.8981922196796337</v>
+        <v>1.881953769950468</v>
       </c>
       <c r="D25" s="5">
         <f t="shared" si="1"/>
-        <v>1.8262242562929061</v>
+        <v>1.8261089708310401</v>
       </c>
       <c r="E25" s="5">
         <f t="shared" si="2"/>
-        <v>1.70120709382151</v>
+        <v>1.7568739680792516</v>
       </c>
       <c r="F25" s="5">
         <f t="shared" si="3"/>
-        <v>1.6322368421052631</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.6366042927903137</v>
+      </c>
+      <c r="G25" s="5">
+        <f t="shared" si="4"/>
+        <v>1.5702531645569622</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>1999</v>
+        <v>2000</v>
       </c>
       <c r="B26" s="5">
-        <v>168.5</v>
+        <v>174.8</v>
       </c>
       <c r="C26" s="5">
         <f t="shared" si="0"/>
-        <v>1.9691632047477743</v>
+        <v>1.956241418764302</v>
       </c>
       <c r="D26" s="5">
         <f t="shared" si="1"/>
-        <v>1.8945044510385756</v>
+        <v>1.8981922196796337</v>
       </c>
       <c r="E26" s="5">
         <f t="shared" si="2"/>
-        <v>1.7648130563798219</v>
+        <v>1.8262242562929061</v>
       </c>
       <c r="F26" s="5">
         <f t="shared" si="3"/>
-        <v>1.6932640949554896</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.70120709382151</v>
+      </c>
+      <c r="G26" s="5">
+        <f t="shared" si="4"/>
+        <v>1.6322368421052631</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="B27" s="5">
-        <v>163.69999999999999</v>
+        <v>168.5</v>
       </c>
       <c r="C27" s="5">
         <f t="shared" si="0"/>
-        <v>2.0269028711056811</v>
+        <v>2.0293827893175074</v>
       </c>
       <c r="D27" s="5">
         <f t="shared" si="1"/>
-        <v>1.9500549786194259</v>
+        <v>1.9691632047477743</v>
       </c>
       <c r="E27" s="5">
         <f t="shared" si="2"/>
-        <v>1.8165607819181429</v>
+        <v>1.8945044510385756</v>
       </c>
       <c r="F27" s="5">
         <f t="shared" si="3"/>
-        <v>1.7429138668295663</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.7648130563798219</v>
+      </c>
+      <c r="G27" s="5">
+        <f t="shared" si="4"/>
+        <v>1.6932640949554896</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="B28" s="5">
-        <v>160.5</v>
+        <v>163.69999999999999</v>
       </c>
       <c r="C28" s="5">
         <f t="shared" si="0"/>
-        <v>2.0673146417445483</v>
+        <v>2.0888882101405013</v>
       </c>
       <c r="D28" s="5">
         <f t="shared" si="1"/>
-        <v>1.9889345794392523</v>
+        <v>2.0269028711056811</v>
       </c>
       <c r="E28" s="5">
         <f t="shared" si="2"/>
-        <v>1.8527788161993768</v>
+        <v>1.9500549786194259</v>
       </c>
       <c r="F28" s="5">
         <f t="shared" si="3"/>
-        <v>1.777663551401869</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.8165607819181429</v>
+      </c>
+      <c r="G28" s="5">
+        <f t="shared" si="4"/>
+        <v>1.7429138668295663</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>1996</v>
+        <v>1997</v>
       </c>
       <c r="B29" s="5">
-        <v>157.1</v>
+        <v>160.5</v>
       </c>
       <c r="C29" s="5">
         <f t="shared" si="0"/>
-        <v>2.1120560152768935</v>
+        <v>2.1305358255451714</v>
       </c>
       <c r="D29" s="5">
         <f t="shared" si="1"/>
-        <v>2.0319796308084022</v>
+        <v>2.0673146417445483</v>
       </c>
       <c r="E29" s="5">
         <f t="shared" si="2"/>
-        <v>1.8928771483131763</v>
+        <v>1.9889345794392523</v>
       </c>
       <c r="F29" s="5">
         <f t="shared" si="3"/>
-        <v>1.8161362189688097</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.8527788161993768</v>
+      </c>
+      <c r="G29" s="5">
+        <f t="shared" si="4"/>
+        <v>1.777663551401869</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>1995</v>
+        <v>1996</v>
       </c>
       <c r="B30" s="5">
-        <v>154</v>
+        <v>157.1</v>
       </c>
       <c r="C30" s="5">
         <f t="shared" si="0"/>
-        <v>2.1545714285714284</v>
+        <v>2.1766454487587525</v>
       </c>
       <c r="D30" s="5">
         <f t="shared" si="1"/>
-        <v>2.072883116883117</v>
+        <v>2.1120560152768935</v>
       </c>
       <c r="E30" s="5">
         <f t="shared" si="2"/>
-        <v>1.9309805194805194</v>
+        <v>2.0319796308084022</v>
       </c>
       <c r="F30" s="5">
         <f t="shared" si="3"/>
-        <v>1.8526948051948051</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.8928771483131763</v>
+      </c>
+      <c r="G30" s="5">
+        <f t="shared" si="4"/>
+        <v>1.8161362189688097</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="B31" s="5">
-        <v>151.5</v>
+        <v>154</v>
       </c>
       <c r="C31" s="5">
         <f t="shared" si="0"/>
-        <v>2.1901254125412541</v>
+        <v>2.2204610389610391</v>
       </c>
       <c r="D31" s="5">
         <f t="shared" si="1"/>
-        <v>2.1070891089108912</v>
+        <v>2.1545714285714284</v>
       </c>
       <c r="E31" s="5">
         <f t="shared" si="2"/>
-        <v>1.9628448844884487</v>
+        <v>2.072883116883117</v>
       </c>
       <c r="F31" s="5">
         <f t="shared" si="3"/>
-        <v>1.8832673267326732</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.9309805194805194</v>
+      </c>
+      <c r="G31" s="5">
+        <f t="shared" si="4"/>
+        <v>1.8526948051948051</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="B32" s="5">
-        <v>149.4</v>
+        <v>151.5</v>
       </c>
       <c r="C32" s="5">
         <f t="shared" si="0"/>
-        <v>2.2209103078982593</v>
+        <v>2.2571023102310233</v>
       </c>
       <c r="D32" s="5">
         <f t="shared" si="1"/>
-        <v>2.1367068273092369</v>
+        <v>2.1901254125412541</v>
       </c>
       <c r="E32" s="5">
         <f t="shared" si="2"/>
-        <v>1.9904350736278444</v>
+        <v>2.1070891089108912</v>
       </c>
       <c r="F32" s="5">
         <f t="shared" si="3"/>
-        <v>1.9097389558232931</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.9628448844884487</v>
+      </c>
+      <c r="G32" s="5">
+        <f t="shared" si="4"/>
+        <v>1.8832673267326732</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="B33" s="5">
-        <v>145.6</v>
+        <v>149.4</v>
       </c>
       <c r="C33" s="5">
         <f t="shared" si="0"/>
-        <v>2.2788736263736262</v>
+        <v>2.2888286479250337</v>
       </c>
       <c r="D33" s="5">
         <f t="shared" si="1"/>
-        <v>2.1924725274725274</v>
+        <v>2.2209103078982593</v>
       </c>
       <c r="E33" s="5">
         <f t="shared" si="2"/>
-        <v>2.0423832417582415</v>
+        <v>2.1367068273092369</v>
       </c>
       <c r="F33" s="5">
         <f t="shared" si="3"/>
-        <v>1.9595810439560439</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.9904350736278444</v>
+      </c>
+      <c r="G33" s="5">
+        <f t="shared" si="4"/>
+        <v>1.9097389558232931</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>1991</v>
+        <v>1992</v>
       </c>
       <c r="B34" s="5">
-        <v>140.6</v>
+        <v>145.6</v>
       </c>
       <c r="C34" s="5">
-        <f t="shared" ref="C34:C65" si="4">$B$2/B34</f>
-        <v>2.3599146514935989</v>
+        <f t="shared" si="0"/>
+        <v>2.3485645604395606</v>
       </c>
       <c r="D34" s="5">
         <f t="shared" si="1"/>
+        <v>2.2788736263736262</v>
+      </c>
+      <c r="E34" s="5">
+        <f t="shared" si="2"/>
+        <v>2.1924725274725274</v>
+      </c>
+      <c r="F34" s="5">
+        <f t="shared" si="3"/>
+        <v>2.0423832417582415</v>
+      </c>
+      <c r="G34" s="5">
+        <f t="shared" si="4"/>
+        <v>1.9595810439560439</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>1991</v>
+      </c>
+      <c r="B35" s="5">
+        <v>140.6</v>
+      </c>
+      <c r="C35" s="5">
+        <f t="shared" si="0"/>
+        <v>2.4320839260312948</v>
+      </c>
+      <c r="D35" s="5">
+        <f t="shared" ref="D35:D66" si="5">$B$3/B35</f>
+        <v>2.3599146514935989</v>
+      </c>
+      <c r="E35" s="5">
+        <f t="shared" si="2"/>
         <v>2.2704409672830725</v>
       </c>
-      <c r="E34" s="5">
-        <f t="shared" si="2"/>
+      <c r="F35" s="5">
+        <f t="shared" si="3"/>
         <v>2.1150142247510666</v>
       </c>
-      <c r="F34" s="5">
-        <f t="shared" si="3"/>
+      <c r="G35" s="5">
+        <f t="shared" si="4"/>
         <v>2.0292674253200569</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36">
         <v>1990</v>
       </c>
-      <c r="B35" s="5">
+      <c r="B36" s="5">
         <v>135</v>
       </c>
-      <c r="C35" s="5">
-        <f t="shared" si="4"/>
+      <c r="C36" s="5">
+        <f t="shared" si="0"/>
+        <v>2.5329703703703705</v>
+      </c>
+      <c r="D36" s="5">
+        <f t="shared" si="5"/>
         <v>2.4578074074074072</v>
       </c>
-      <c r="D35" s="5">
-        <f t="shared" si="1"/>
+      <c r="E36" s="5">
+        <f t="shared" si="2"/>
         <v>2.3646222222222222</v>
       </c>
-      <c r="E35" s="5">
-        <f t="shared" si="2"/>
+      <c r="F36" s="5">
+        <f t="shared" si="3"/>
         <v>2.2027481481481481</v>
       </c>
-      <c r="F35" s="5">
-        <f t="shared" si="3"/>
+      <c r="G36" s="5">
+        <f t="shared" si="4"/>
         <v>2.1134444444444442</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37">
         <v>1989</v>
       </c>
-      <c r="B36" s="5">
+      <c r="B37" s="5">
         <v>128</v>
       </c>
-      <c r="C36" s="5">
-        <f t="shared" si="4"/>
+      <c r="C37" s="5">
+        <f t="shared" si="0"/>
+        <v>2.6714921875000002</v>
+      </c>
+      <c r="D37" s="5">
+        <f t="shared" si="5"/>
         <v>2.5922187499999998</v>
       </c>
-      <c r="D36" s="5">
-        <f t="shared" si="1"/>
+      <c r="E37" s="5">
+        <f t="shared" si="2"/>
         <v>2.4939374999999999</v>
       </c>
-      <c r="E36" s="5">
-        <f t="shared" si="2"/>
+      <c r="F37" s="5">
+        <f t="shared" si="3"/>
         <v>2.3232109374999999</v>
       </c>
-      <c r="F36" s="5">
-        <f t="shared" si="3"/>
+      <c r="G37" s="5">
+        <f t="shared" si="4"/>
         <v>2.2290234375</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38">
         <v>1988</v>
       </c>
-      <c r="B37" s="5">
+      <c r="B38" s="5">
         <v>121.9</v>
       </c>
-      <c r="C37" s="5">
-        <f t="shared" si="4"/>
+      <c r="C38" s="5">
+        <f t="shared" si="0"/>
+        <v>2.8051763740771123</v>
+      </c>
+      <c r="D38" s="5">
+        <f t="shared" si="5"/>
         <v>2.7219360131255126</v>
       </c>
-      <c r="D37" s="5">
-        <f t="shared" si="1"/>
+      <c r="E38" s="5">
+        <f t="shared" si="2"/>
         <v>2.6187366694011485</v>
       </c>
-      <c r="E37" s="5">
-        <f t="shared" si="2"/>
+      <c r="F38" s="5">
+        <f t="shared" si="3"/>
         <v>2.439466776045939</v>
       </c>
-      <c r="F37" s="5">
-        <f t="shared" si="3"/>
+      <c r="G38" s="5">
+        <f t="shared" si="4"/>
         <v>2.340566037735849</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39">
         <v>1987</v>
       </c>
-      <c r="B38" s="5">
+      <c r="B39" s="5">
         <v>116.5</v>
       </c>
-      <c r="C38" s="5">
-        <f t="shared" si="4"/>
+      <c r="C39" s="5">
+        <f t="shared" si="0"/>
+        <v>2.9352017167381974</v>
+      </c>
+      <c r="D39" s="5">
+        <f t="shared" si="5"/>
         <v>2.8481030042918452</v>
       </c>
-      <c r="D38" s="5">
-        <f t="shared" si="1"/>
+      <c r="E39" s="5">
+        <f t="shared" si="2"/>
         <v>2.7401201716738197</v>
       </c>
-      <c r="E38" s="5">
-        <f t="shared" si="2"/>
+      <c r="F39" s="5">
+        <f t="shared" si="3"/>
         <v>2.5525407725321885</v>
       </c>
-      <c r="F38" s="5">
-        <f t="shared" si="3"/>
+      <c r="G39" s="5">
+        <f t="shared" si="4"/>
         <v>2.4490557939914162</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40">
         <v>1986</v>
       </c>
-      <c r="B39" s="5">
+      <c r="B40" s="5">
         <v>112</v>
       </c>
-      <c r="C39" s="5">
-        <f t="shared" si="4"/>
+      <c r="C40" s="5">
+        <f t="shared" si="0"/>
+        <v>3.053133928571429</v>
+      </c>
+      <c r="D40" s="5">
+        <f t="shared" si="5"/>
         <v>2.9625357142857141</v>
       </c>
-      <c r="D39" s="5">
-        <f t="shared" si="1"/>
+      <c r="E40" s="5">
+        <f t="shared" si="2"/>
         <v>2.8502142857142858</v>
       </c>
-      <c r="E39" s="5">
-        <f t="shared" si="2"/>
+      <c r="F40" s="5">
+        <f t="shared" si="3"/>
         <v>2.6550982142857142</v>
       </c>
-      <c r="F39" s="5">
-        <f t="shared" si="3"/>
+      <c r="G40" s="5">
+        <f t="shared" si="4"/>
         <v>2.5474553571428573</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41">
         <v>1985</v>
       </c>
-      <c r="B40" s="5">
+      <c r="B41" s="5">
         <v>108.6</v>
       </c>
-      <c r="C40" s="5">
-        <f t="shared" si="4"/>
+      <c r="C41" s="5">
+        <f t="shared" si="0"/>
+        <v>3.1487200736648253</v>
+      </c>
+      <c r="D41" s="5">
+        <f t="shared" si="5"/>
         <v>3.0552854511970535</v>
       </c>
-      <c r="D40" s="5">
-        <f t="shared" si="1"/>
+      <c r="E41" s="5">
+        <f t="shared" si="2"/>
         <v>2.939447513812155</v>
       </c>
-      <c r="E40" s="5">
-        <f t="shared" si="2"/>
+      <c r="F41" s="5">
+        <f t="shared" si="3"/>
         <v>2.7382228360957641</v>
       </c>
-      <c r="F40" s="5">
-        <f t="shared" si="3"/>
+      <c r="G41" s="5">
+        <f t="shared" si="4"/>
         <v>2.6272099447513813</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42">
         <v>1984</v>
       </c>
-      <c r="B41" s="5">
+      <c r="B42" s="5">
         <v>103.8</v>
       </c>
-      <c r="C41" s="5">
-        <f t="shared" si="4"/>
+      <c r="C42" s="5">
+        <f t="shared" si="0"/>
+        <v>3.2943256262042393</v>
+      </c>
+      <c r="D42" s="5">
+        <f t="shared" si="5"/>
         <v>3.1965703275529864</v>
       </c>
-      <c r="D41" s="5">
-        <f t="shared" si="1"/>
+      <c r="E42" s="5">
+        <f t="shared" si="2"/>
         <v>3.0753757225433525</v>
       </c>
-      <c r="E41" s="5">
-        <f t="shared" si="2"/>
+      <c r="F42" s="5">
+        <f t="shared" si="3"/>
         <v>2.8648458574181115</v>
       </c>
-      <c r="F41" s="5">
-        <f t="shared" si="3"/>
+      <c r="G42" s="5">
+        <f t="shared" si="4"/>
         <v>2.748699421965318</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43">
         <v>1983</v>
       </c>
-      <c r="B42" s="5">
+      <c r="B43" s="5">
         <v>98.9</v>
       </c>
-      <c r="C42" s="5">
-        <f t="shared" si="4"/>
+      <c r="C43" s="5">
+        <f t="shared" si="0"/>
+        <v>3.4575429726996969</v>
+      </c>
+      <c r="D43" s="5">
+        <f t="shared" si="5"/>
         <v>3.3549443882709804</v>
       </c>
-      <c r="D42" s="5">
-        <f t="shared" si="1"/>
+      <c r="E43" s="5">
+        <f t="shared" si="2"/>
         <v>3.2277451971688573</v>
       </c>
-      <c r="E42" s="5">
-        <f t="shared" si="2"/>
+      <c r="F43" s="5">
+        <f t="shared" si="3"/>
         <v>3.0067846309403432</v>
       </c>
-      <c r="F42" s="5">
-        <f t="shared" si="3"/>
+      <c r="G43" s="5">
+        <f t="shared" si="4"/>
         <v>2.8848837209302323</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44">
         <v>1982</v>
       </c>
-      <c r="B43" s="5">
+      <c r="B44" s="5">
         <v>97.3</v>
       </c>
-      <c r="C43" s="5">
-        <f t="shared" si="4"/>
+      <c r="C44" s="5">
+        <f t="shared" si="0"/>
+        <v>3.5143987667009253</v>
+      </c>
+      <c r="D44" s="5">
+        <f t="shared" si="5"/>
         <v>3.4101130524152103</v>
       </c>
-      <c r="D43" s="5">
-        <f t="shared" si="1"/>
+      <c r="E44" s="5">
+        <f t="shared" si="2"/>
         <v>3.2808221993833504</v>
       </c>
-      <c r="E43" s="5">
-        <f t="shared" si="2"/>
+      <c r="F44" s="5">
+        <f t="shared" si="3"/>
         <v>3.0562281603288795</v>
       </c>
-      <c r="F43" s="5">
-        <f t="shared" si="3"/>
+      <c r="G44" s="5">
+        <f t="shared" si="4"/>
         <v>2.9323227132579652</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45">
         <v>1981</v>
       </c>
-      <c r="B44" s="5">
+      <c r="B45" s="5">
         <v>91.4</v>
       </c>
-      <c r="C44" s="5">
-        <f t="shared" si="4"/>
+      <c r="C45" s="5">
+        <f t="shared" si="0"/>
+        <v>3.7412582056892778</v>
+      </c>
+      <c r="D45" s="5">
+        <f t="shared" si="5"/>
         <v>3.6302407002188177</v>
       </c>
-      <c r="D44" s="5">
-        <f t="shared" si="1"/>
+      <c r="E45" s="5">
+        <f t="shared" si="2"/>
         <v>3.492603938730853</v>
       </c>
-      <c r="E44" s="5">
-        <f t="shared" si="2"/>
+      <c r="F45" s="5">
+        <f t="shared" si="3"/>
         <v>3.2535120350109406</v>
       </c>
-      <c r="F44" s="5">
-        <f t="shared" si="3"/>
+      <c r="G45" s="5">
+        <f t="shared" si="4"/>
         <v>3.1216083150984679</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46">
         <v>1980</v>
       </c>
-      <c r="B45" s="5">
+      <c r="B46" s="5">
         <v>82.4</v>
       </c>
-      <c r="C45" s="5">
-        <f t="shared" si="4"/>
+      <c r="C46" s="5">
+        <f t="shared" si="0"/>
+        <v>4.1498907766990287</v>
+      </c>
+      <c r="D46" s="5">
+        <f t="shared" si="5"/>
         <v>4.0267475728155331</v>
       </c>
-      <c r="D45" s="5">
-        <f t="shared" si="1"/>
+      <c r="E46" s="5">
+        <f t="shared" si="2"/>
         <v>3.874077669902912</v>
       </c>
-      <c r="E45" s="5">
-        <f t="shared" si="2"/>
+      <c r="F46" s="5">
+        <f t="shared" si="3"/>
         <v>3.6088713592233006</v>
       </c>
-      <c r="F45" s="5">
-        <f t="shared" si="3"/>
+      <c r="G46" s="5">
+        <f t="shared" si="4"/>
         <v>3.4625606796116504</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47">
         <v>1979</v>
       </c>
-      <c r="B46" s="5">
+      <c r="B47" s="5">
         <v>71.3</v>
       </c>
-      <c r="C46" s="5">
-        <f t="shared" si="4"/>
+      <c r="C47" s="5">
+        <f t="shared" si="0"/>
+        <v>4.7959467040673216</v>
+      </c>
+      <c r="D47" s="5">
+        <f t="shared" si="5"/>
         <v>4.6536325385694246</v>
       </c>
-      <c r="D46" s="5">
-        <f t="shared" si="1"/>
+      <c r="E47" s="5">
+        <f t="shared" si="2"/>
         <v>4.4771949509116409</v>
       </c>
-      <c r="E46" s="5">
-        <f t="shared" si="2"/>
+      <c r="F47" s="5">
+        <f t="shared" si="3"/>
         <v>4.1707012622720896</v>
       </c>
-      <c r="F46" s="5">
-        <f t="shared" si="3"/>
+      <c r="G47" s="5">
+        <f t="shared" si="4"/>
         <v>4.0016129032258068</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48">
         <v>1978</v>
       </c>
-      <c r="B47" s="5">
+      <c r="B48" s="5">
         <v>64.400000000000006</v>
       </c>
-      <c r="C47" s="5">
-        <f t="shared" si="4"/>
+      <c r="C48" s="5">
+        <f t="shared" si="0"/>
+        <v>5.3097981366459628</v>
+      </c>
+      <c r="D48" s="5">
+        <f t="shared" si="5"/>
         <v>5.1522360248447194</v>
       </c>
-      <c r="D47" s="5">
-        <f t="shared" si="1"/>
+      <c r="E48" s="5">
+        <f t="shared" si="2"/>
         <v>4.9568944099378873</v>
       </c>
-      <c r="E47" s="5">
-        <f t="shared" si="2"/>
+      <c r="F48" s="5">
+        <f t="shared" si="3"/>
         <v>4.6175621118012415</v>
       </c>
-      <c r="F47" s="5">
-        <f t="shared" si="3"/>
+      <c r="G48" s="5">
+        <f t="shared" si="4"/>
         <v>4.430357142857142</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49">
         <v>1977</v>
       </c>
-      <c r="B48" s="5">
+      <c r="B49" s="5">
         <v>59.5</v>
       </c>
-      <c r="C48" s="5">
-        <f t="shared" si="4"/>
+      <c r="C49" s="5">
+        <f t="shared" si="0"/>
+        <v>5.7470756302521009</v>
+      </c>
+      <c r="D49" s="5">
+        <f t="shared" si="5"/>
         <v>5.5765378151260503</v>
       </c>
-      <c r="D48" s="5">
-        <f t="shared" si="1"/>
+      <c r="E49" s="5">
+        <f t="shared" si="2"/>
         <v>5.3651092436974785</v>
       </c>
-      <c r="E48" s="5">
-        <f t="shared" si="2"/>
+      <c r="F49" s="5">
+        <f t="shared" si="3"/>
         <v>4.9978319327731091</v>
       </c>
-      <c r="F48" s="5">
-        <f t="shared" si="3"/>
+      <c r="G49" s="5">
+        <f t="shared" si="4"/>
         <v>4.7952100840336138</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50">
         <v>1976</v>
       </c>
-      <c r="B49" s="5">
+      <c r="B50" s="5">
         <v>55.6</v>
       </c>
-      <c r="C49" s="5">
-        <f t="shared" si="4"/>
+      <c r="C50" s="5">
+        <f t="shared" si="0"/>
+        <v>6.1501978417266185</v>
+      </c>
+      <c r="D50" s="5">
+        <f t="shared" si="5"/>
         <v>5.9676978417266184</v>
       </c>
-      <c r="D49" s="5">
-        <f t="shared" si="1"/>
+      <c r="E50" s="5">
+        <f t="shared" si="2"/>
         <v>5.741438848920863</v>
       </c>
-      <c r="E49" s="5">
-        <f t="shared" si="2"/>
+      <c r="F50" s="5">
+        <f t="shared" si="3"/>
         <v>5.3483992805755394</v>
       </c>
-      <c r="F49" s="5">
-        <f t="shared" si="3"/>
+      <c r="G50" s="5">
+        <f t="shared" si="4"/>
         <v>5.1315647482014386</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51">
         <v>1975</v>
       </c>
-      <c r="B50" s="5">
+      <c r="B51" s="5">
         <v>52.3</v>
       </c>
-      <c r="C50" s="5">
-        <f t="shared" si="4"/>
+      <c r="C51" s="5">
+        <f t="shared" si="0"/>
+        <v>6.5382600382409182</v>
+      </c>
+      <c r="D51" s="5">
+        <f t="shared" si="5"/>
         <v>6.3442447418738048</v>
       </c>
-      <c r="D50" s="5">
-        <f t="shared" si="1"/>
+      <c r="E51" s="5">
+        <f t="shared" si="2"/>
         <v>6.1037093690248572</v>
       </c>
-      <c r="E50" s="5">
-        <f t="shared" si="2"/>
+      <c r="F51" s="5">
+        <f t="shared" si="3"/>
         <v>5.6858699808795414</v>
       </c>
-      <c r="F50" s="5">
-        <f t="shared" si="3"/>
+      <c r="G51" s="5">
+        <f t="shared" si="4"/>
         <v>5.4553537284894844</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52">
         <v>1974</v>
       </c>
-      <c r="B51" s="5">
+      <c r="B52" s="5">
         <v>47.4</v>
       </c>
-      <c r="C51" s="5">
-        <f t="shared" si="4"/>
+      <c r="C52" s="5">
+        <f t="shared" si="0"/>
+        <v>7.2141561181434604</v>
+      </c>
+      <c r="D52" s="5">
+        <f t="shared" si="5"/>
         <v>7.0000843881856536</v>
       </c>
-      <c r="D51" s="5">
-        <f t="shared" si="1"/>
+      <c r="E52" s="5">
+        <f t="shared" si="2"/>
         <v>6.7346835443037971</v>
       </c>
-      <c r="E51" s="5">
-        <f t="shared" si="2"/>
+      <c r="F52" s="5">
+        <f t="shared" si="3"/>
         <v>6.2736497890295357</v>
       </c>
-      <c r="F51" s="5">
-        <f t="shared" si="3"/>
+      <c r="G52" s="5">
+        <f t="shared" si="4"/>
         <v>6.0193037974683543</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53">
         <v>1973</v>
       </c>
-      <c r="B52" s="5">
+      <c r="B53" s="5">
         <v>43</v>
       </c>
-      <c r="C52" s="5">
-        <f t="shared" si="4"/>
+      <c r="C53" s="5">
+        <f t="shared" si="0"/>
+        <v>7.9523488372093025</v>
+      </c>
+      <c r="D53" s="5">
+        <f t="shared" si="5"/>
         <v>7.7163720930232556</v>
       </c>
-      <c r="D52" s="5">
-        <f t="shared" si="1"/>
+      <c r="E53" s="5">
+        <f t="shared" si="2"/>
         <v>7.4238139534883718</v>
       </c>
-      <c r="E52" s="5">
-        <f t="shared" si="2"/>
+      <c r="F53" s="5">
+        <f t="shared" si="3"/>
         <v>6.9156046511627904</v>
       </c>
-      <c r="F52" s="5">
-        <f t="shared" si="3"/>
+      <c r="G53" s="5">
+        <f t="shared" si="4"/>
         <v>6.6352325581395348</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54">
         <v>1972</v>
       </c>
-      <c r="B53" s="5">
+      <c r="B54" s="5">
         <v>40.6</v>
       </c>
-      <c r="C53" s="5">
-        <f t="shared" si="4"/>
+      <c r="C54" s="5">
+        <f t="shared" si="0"/>
+        <v>8.4224384236453211</v>
+      </c>
+      <c r="D54" s="5">
+        <f t="shared" si="5"/>
         <v>8.1725123152709358</v>
       </c>
-      <c r="D53" s="5">
-        <f t="shared" si="1"/>
+      <c r="E54" s="5">
+        <f t="shared" si="2"/>
         <v>7.8626600985221673</v>
       </c>
-      <c r="E53" s="5">
-        <f t="shared" si="2"/>
+      <c r="F54" s="5">
+        <f t="shared" si="3"/>
         <v>7.3244088669950731</v>
       </c>
-      <c r="F53" s="5">
-        <f t="shared" si="3"/>
+      <c r="G54" s="5">
+        <f t="shared" si="4"/>
         <v>7.0274630541871916</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55">
         <v>1971</v>
       </c>
-      <c r="B54" s="5">
+      <c r="B55" s="5">
         <v>39.299999999999997</v>
       </c>
-      <c r="C54" s="5">
-        <f t="shared" si="4"/>
+      <c r="C55" s="5">
+        <f t="shared" si="0"/>
+        <v>8.7010432569974565</v>
+      </c>
+      <c r="D55" s="5">
+        <f t="shared" si="5"/>
         <v>8.4428498727735377</v>
       </c>
-      <c r="D54" s="5">
-        <f t="shared" si="1"/>
+      <c r="E55" s="5">
+        <f t="shared" si="2"/>
         <v>8.1227480916030537</v>
       </c>
-      <c r="E54" s="5">
-        <f t="shared" si="2"/>
+      <c r="F55" s="5">
+        <f t="shared" si="3"/>
         <v>7.5666921119592878</v>
       </c>
-      <c r="F54" s="5">
-        <f t="shared" si="3"/>
+      <c r="G55" s="5">
+        <f t="shared" si="4"/>
         <v>7.2599236641221383</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56">
         <v>1970</v>
       </c>
-      <c r="B55" s="5">
+      <c r="B56" s="5">
         <v>37.9</v>
       </c>
-      <c r="C55" s="5">
-        <f t="shared" si="4"/>
+      <c r="C56" s="5">
+        <f t="shared" si="0"/>
+        <v>9.0224538258575215</v>
+      </c>
+      <c r="D56" s="5">
+        <f t="shared" si="5"/>
         <v>8.7547229551451178</v>
       </c>
-      <c r="D55" s="5">
-        <f t="shared" si="1"/>
+      <c r="E56" s="5">
+        <f t="shared" si="2"/>
         <v>8.4227968337730879</v>
       </c>
-      <c r="E55" s="5">
-        <f t="shared" si="2"/>
+      <c r="F56" s="5">
+        <f t="shared" si="3"/>
         <v>7.8462005277044851</v>
       </c>
-      <c r="F55" s="5">
-        <f t="shared" si="3"/>
+      <c r="G56" s="5">
+        <f t="shared" si="4"/>
         <v>7.5281002638522434</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57">
         <v>1969</v>
       </c>
-      <c r="B56" s="5">
+      <c r="B57" s="5">
         <v>36.1</v>
       </c>
-      <c r="C56" s="5">
-        <f t="shared" si="4"/>
+      <c r="C57" s="5">
+        <f t="shared" si="0"/>
+        <v>9.4723268698060945</v>
+      </c>
+      <c r="D57" s="5">
+        <f t="shared" si="5"/>
         <v>9.1912465373961201</v>
       </c>
-      <c r="D56" s="5">
-        <f t="shared" si="1"/>
+      <c r="E57" s="5">
+        <f t="shared" si="2"/>
         <v>8.8427700831024918</v>
       </c>
-      <c r="E56" s="5">
-        <f t="shared" si="2"/>
+      <c r="F57" s="5">
+        <f t="shared" si="3"/>
         <v>8.2374238227146801</v>
       </c>
-      <c r="F56" s="5">
-        <f t="shared" si="3"/>
+      <c r="G57" s="5">
+        <f t="shared" si="4"/>
         <v>7.9034626038781157</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58">
         <v>1968</v>
       </c>
-      <c r="B57" s="5">
+      <c r="B58" s="5">
         <v>34.4</v>
       </c>
-      <c r="C57" s="5">
-        <f t="shared" si="4"/>
+      <c r="C58" s="5">
+        <f t="shared" si="0"/>
+        <v>9.9404360465116284</v>
+      </c>
+      <c r="D58" s="5">
+        <f t="shared" si="5"/>
         <v>9.6454651162790697</v>
       </c>
-      <c r="D57" s="5">
-        <f t="shared" si="1"/>
+      <c r="E58" s="5">
+        <f t="shared" si="2"/>
         <v>9.2797674418604643</v>
       </c>
-      <c r="E57" s="5">
-        <f t="shared" si="2"/>
+      <c r="F58" s="5">
+        <f t="shared" si="3"/>
         <v>8.6445058139534883</v>
       </c>
-      <c r="F57" s="5">
-        <f t="shared" si="3"/>
+      <c r="G58" s="5">
+        <f t="shared" si="4"/>
         <v>8.2940406976744185</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59">
         <v>1967</v>
       </c>
-      <c r="B58" s="5">
+      <c r="B59" s="5">
         <v>33</v>
       </c>
-      <c r="C58" s="5">
-        <f t="shared" si="4"/>
+      <c r="C59" s="5">
+        <f t="shared" si="0"/>
+        <v>10.362151515151515</v>
+      </c>
+      <c r="D59" s="5">
+        <f t="shared" si="5"/>
         <v>10.054666666666666</v>
       </c>
-      <c r="D58" s="5">
-        <f t="shared" si="1"/>
+      <c r="E59" s="5">
+        <f t="shared" si="2"/>
         <v>9.6734545454545451</v>
       </c>
-      <c r="E58" s="5">
-        <f t="shared" si="2"/>
+      <c r="F59" s="5">
+        <f t="shared" si="3"/>
         <v>9.0112424242424236</v>
       </c>
-      <c r="F58" s="5">
-        <f t="shared" si="3"/>
+      <c r="G59" s="5">
+        <f t="shared" si="4"/>
         <v>8.6459090909090914</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60">
         <v>1966</v>
       </c>
-      <c r="B59" s="5">
+      <c r="B60" s="5">
         <v>32.200000000000003</v>
       </c>
-      <c r="C59" s="5">
-        <f t="shared" si="4"/>
+      <c r="C60" s="5">
+        <f t="shared" si="0"/>
+        <v>10.619596273291926</v>
+      </c>
+      <c r="D60" s="5">
+        <f t="shared" si="5"/>
         <v>10.304472049689439</v>
       </c>
-      <c r="D59" s="5">
-        <f t="shared" si="1"/>
+      <c r="E60" s="5">
+        <f t="shared" si="2"/>
         <v>9.9137888198757746</v>
       </c>
-      <c r="E59" s="5">
-        <f t="shared" si="2"/>
+      <c r="F60" s="5">
+        <f t="shared" si="3"/>
         <v>9.2351242236024831</v>
       </c>
-      <c r="F59" s="5">
-        <f t="shared" si="3"/>
+      <c r="G60" s="5">
+        <f t="shared" si="4"/>
         <v>8.860714285714284</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61">
         <v>1965</v>
       </c>
-      <c r="B60" s="5">
+      <c r="B61" s="5">
         <v>31.5</v>
       </c>
-      <c r="C60" s="5">
-        <f t="shared" si="4"/>
+      <c r="C61" s="5">
+        <f t="shared" si="0"/>
+        <v>10.855587301587303</v>
+      </c>
+      <c r="D61" s="5">
+        <f t="shared" si="5"/>
         <v>10.533460317460317</v>
       </c>
-      <c r="D60" s="5">
-        <f t="shared" si="1"/>
+      <c r="E61" s="5">
+        <f t="shared" si="2"/>
         <v>10.134095238095238</v>
       </c>
-      <c r="E60" s="5">
-        <f t="shared" si="2"/>
+      <c r="F61" s="5">
+        <f t="shared" si="3"/>
         <v>9.4403492063492056</v>
       </c>
-      <c r="F60" s="5">
-        <f t="shared" si="3"/>
+      <c r="G61" s="5">
+        <f t="shared" si="4"/>
         <v>9.0576190476190472</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62">
         <v>1964</v>
       </c>
-      <c r="B61" s="5">
+      <c r="B62" s="5">
         <v>31</v>
       </c>
-      <c r="C61" s="5">
-        <f t="shared" si="4"/>
+      <c r="C62" s="5">
+        <f t="shared" si="0"/>
+        <v>11.03067741935484</v>
+      </c>
+      <c r="D62" s="5">
+        <f t="shared" si="5"/>
         <v>10.703354838709677</v>
       </c>
-      <c r="D61" s="5">
-        <f t="shared" si="1"/>
+      <c r="E62" s="5">
+        <f t="shared" si="2"/>
         <v>10.297548387096773</v>
       </c>
-      <c r="E61" s="5">
-        <f t="shared" si="2"/>
+      <c r="F62" s="5">
+        <f t="shared" si="3"/>
         <v>9.5926129032258061</v>
       </c>
-      <c r="F61" s="5">
-        <f t="shared" si="3"/>
+      <c r="G62" s="5">
+        <f t="shared" si="4"/>
         <v>9.2037096774193543</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63">
         <v>1963</v>
       </c>
-      <c r="B62" s="5">
+      <c r="B63" s="5">
         <v>30.4</v>
       </c>
-      <c r="C62" s="5">
-        <f t="shared" si="4"/>
+      <c r="C63" s="5">
+        <f t="shared" si="0"/>
+        <v>11.248388157894738</v>
+      </c>
+      <c r="D63" s="5">
+        <f t="shared" si="5"/>
         <v>10.914605263157894</v>
       </c>
-      <c r="D62" s="5">
-        <f t="shared" si="1"/>
+      <c r="E63" s="5">
+        <f t="shared" si="2"/>
         <v>10.500789473684211</v>
       </c>
-      <c r="E62" s="5">
-        <f t="shared" si="2"/>
+      <c r="F63" s="5">
+        <f t="shared" si="3"/>
         <v>9.7819407894736834</v>
       </c>
-      <c r="F62" s="5">
-        <f t="shared" si="3"/>
+      <c r="G63" s="5">
+        <f t="shared" si="4"/>
         <v>9.3853618421052634</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64">
         <v>1962</v>
       </c>
-      <c r="B63" s="5">
+      <c r="B64" s="5">
         <v>29.9</v>
       </c>
-      <c r="C63" s="5">
-        <f t="shared" si="4"/>
+      <c r="C64" s="5">
+        <f t="shared" si="0"/>
+        <v>11.436488294314383</v>
+      </c>
+      <c r="D64" s="5">
+        <f t="shared" si="5"/>
         <v>11.097123745819397</v>
       </c>
-      <c r="D63" s="5">
-        <f t="shared" si="1"/>
+      <c r="E64" s="5">
+        <f t="shared" si="2"/>
         <v>10.67638795986622</v>
       </c>
-      <c r="E63" s="5">
-        <f t="shared" si="2"/>
+      <c r="F64" s="5">
+        <f t="shared" si="3"/>
         <v>9.945518394648829</v>
       </c>
-      <c r="F63" s="5">
-        <f t="shared" si="3"/>
+      <c r="G64" s="5">
+        <f t="shared" si="4"/>
         <v>9.542307692307693</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65">
         <v>1961</v>
       </c>
-      <c r="B64" s="5">
+      <c r="B65" s="5">
         <v>29.5</v>
       </c>
-      <c r="C64" s="5">
-        <f t="shared" si="4"/>
+      <c r="C65" s="5">
+        <f t="shared" si="0"/>
+        <v>11.591559322033898</v>
+      </c>
+      <c r="D65" s="5">
+        <f t="shared" si="5"/>
         <v>11.247593220338983</v>
       </c>
-      <c r="D64" s="5">
-        <f t="shared" si="1"/>
+      <c r="E65" s="5">
+        <f t="shared" si="2"/>
         <v>10.82115254237288</v>
       </c>
-      <c r="E64" s="5">
-        <f t="shared" si="2"/>
+      <c r="F65" s="5">
+        <f t="shared" si="3"/>
         <v>10.080372881355931</v>
       </c>
-      <c r="F64" s="5">
-        <f t="shared" si="3"/>
+      <c r="G65" s="5">
+        <f t="shared" si="4"/>
         <v>9.6716949152542373</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66">
         <v>1960</v>
       </c>
-      <c r="B65" s="5">
+      <c r="B66" s="5">
         <v>29.2</v>
       </c>
-      <c r="C65" s="5">
-        <f t="shared" si="4"/>
+      <c r="C66" s="5">
+        <f t="shared" si="0"/>
+        <v>11.710650684931508</v>
+      </c>
+      <c r="D66" s="5">
+        <f t="shared" si="5"/>
         <v>11.363150684931506</v>
       </c>
-      <c r="D65" s="5">
-        <f t="shared" si="1"/>
+      <c r="E66" s="5">
+        <f t="shared" si="2"/>
         <v>10.932328767123288</v>
       </c>
-      <c r="E65" s="5">
-        <f t="shared" si="2"/>
+      <c r="F66" s="5">
+        <f t="shared" si="3"/>
         <v>10.183938356164383</v>
       </c>
-      <c r="F65" s="5">
-        <f t="shared" si="3"/>
+      <c r="G66" s="5">
+        <f t="shared" si="4"/>
         <v>9.7710616438356173</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67">
         <v>1959</v>
       </c>
-      <c r="B66" s="5">
+      <c r="B67" s="5">
         <v>28.6</v>
       </c>
-      <c r="C66" s="5">
-        <f t="shared" ref="C66:C97" si="5">$B$2/B66</f>
+      <c r="C67" s="5">
+        <f t="shared" si="0"/>
+        <v>11.956328671328672</v>
+      </c>
+      <c r="D67" s="5">
+        <f t="shared" ref="D67:D71" si="6">$B$3/B67</f>
         <v>11.60153846153846</v>
       </c>
-      <c r="D66" s="5">
-        <f t="shared" si="1"/>
+      <c r="E67" s="5">
+        <f t="shared" si="2"/>
         <v>11.161678321678322</v>
       </c>
-      <c r="E66" s="5">
-        <f t="shared" si="2"/>
+      <c r="F67" s="5">
+        <f t="shared" si="3"/>
         <v>10.397587412587411</v>
       </c>
-      <c r="F66" s="5">
-        <f t="shared" si="3"/>
+      <c r="G67" s="5">
+        <f t="shared" si="4"/>
         <v>9.9760489510489503</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68">
         <v>1958</v>
       </c>
-      <c r="B67" s="5">
+      <c r="B68" s="5">
         <v>28.1</v>
       </c>
-      <c r="C67" s="5">
-        <f t="shared" si="5"/>
-        <v>11.807971530249109</v>
-      </c>
-      <c r="D67" s="5">
-        <f t="shared" ref="D67:D70" si="6">$B$3/B67</f>
-        <v>11.360284697508895</v>
-      </c>
-      <c r="E67" s="5">
-        <f t="shared" ref="E67:E70" si="7">$B$4/B67</f>
-        <v>10.582597864768681</v>
-      </c>
-      <c r="F67" s="5">
-        <f t="shared" ref="F67:F70" si="8">$B$5/B67</f>
-        <v>10.153558718861209</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68">
-        <v>1957</v>
-      </c>
-      <c r="B68" s="5">
-        <v>27.1</v>
-      </c>
       <c r="C68" s="5">
-        <f t="shared" si="5"/>
-        <v>12.243690036900368</v>
+        <f t="shared" ref="C68:C71" si="7">$B$2/B68</f>
+        <v>12.169074733096085</v>
       </c>
       <c r="D68" s="5">
         <f t="shared" si="6"/>
-        <v>11.779483394833948</v>
+        <v>11.807971530249109</v>
       </c>
       <c r="E68" s="5">
+        <f t="shared" ref="E68:E71" si="8">$B$4/B68</f>
+        <v>11.360284697508895</v>
+      </c>
+      <c r="F68" s="5">
+        <f t="shared" ref="F68:F71" si="9">$B$5/B68</f>
+        <v>10.582597864768681</v>
+      </c>
+      <c r="G68" s="5">
+        <f t="shared" ref="G68:G71" si="10">$B$6/B68</f>
+        <v>10.153558718861209</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>1957</v>
+      </c>
+      <c r="B69" s="5">
+        <v>27.1</v>
+      </c>
+      <c r="C69" s="5">
         <f t="shared" si="7"/>
-        <v>10.973099630996309</v>
-      </c>
-      <c r="F68" s="5">
-        <f t="shared" si="8"/>
-        <v>10.528228782287822</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69">
-        <v>1956</v>
-      </c>
-      <c r="B69" s="5">
-        <v>26.2</v>
-      </c>
-      <c r="C69" s="5">
-        <f t="shared" si="5"/>
-        <v>12.664274809160304</v>
+        <v>12.618118081180812</v>
       </c>
       <c r="D69" s="5">
         <f t="shared" si="6"/>
-        <v>12.18412213740458</v>
+        <v>12.243690036900368</v>
       </c>
       <c r="E69" s="5">
+        <f t="shared" si="8"/>
+        <v>11.779483394833948</v>
+      </c>
+      <c r="F69" s="5">
+        <f t="shared" si="9"/>
+        <v>10.973099630996309</v>
+      </c>
+      <c r="G69" s="5">
+        <f t="shared" si="10"/>
+        <v>10.528228782287822</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>1956</v>
+      </c>
+      <c r="B70" s="5">
+        <v>26.2</v>
+      </c>
+      <c r="C70" s="5">
         <f t="shared" si="7"/>
-        <v>11.350038167938932</v>
-      </c>
-      <c r="F69" s="5">
-        <f t="shared" si="8"/>
-        <v>10.889885496183206</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70">
-        <v>1955</v>
-      </c>
-      <c r="B70" s="5">
-        <v>25.7</v>
-      </c>
-      <c r="C70" s="5">
-        <f t="shared" si="5"/>
-        <v>12.910661478599222</v>
+        <v>13.051564885496184</v>
       </c>
       <c r="D70" s="5">
         <f t="shared" si="6"/>
+        <v>12.664274809160304</v>
+      </c>
+      <c r="E70" s="5">
+        <f t="shared" si="8"/>
+        <v>12.18412213740458</v>
+      </c>
+      <c r="F70" s="5">
+        <f t="shared" si="9"/>
+        <v>11.350038167938932</v>
+      </c>
+      <c r="G70" s="5">
+        <f t="shared" si="10"/>
+        <v>10.889885496183206</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>1955</v>
+      </c>
+      <c r="B71" s="5">
+        <v>25.7</v>
+      </c>
+      <c r="C71" s="5">
+        <f t="shared" si="7"/>
+        <v>13.305486381322959</v>
+      </c>
+      <c r="D71" s="5">
+        <f t="shared" si="6"/>
+        <v>12.910661478599222</v>
+      </c>
+      <c r="E71" s="5">
+        <f t="shared" si="8"/>
         <v>12.421167315175097</v>
       </c>
-      <c r="E70" s="5">
-        <f t="shared" si="7"/>
+      <c r="F71" s="5">
+        <f t="shared" si="9"/>
         <v>11.570856031128404</v>
       </c>
-      <c r="F70" s="5">
-        <f t="shared" si="8"/>
+      <c r="G71" s="5">
+        <f t="shared" si="10"/>
         <v>11.101750972762646</v>
       </c>
     </row>

</xml_diff>